<commit_message>
added all 5 spiders for the real websites finally lol
</commit_message>
<xml_diff>
--- a/conference_data.xlsx
+++ b/conference_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -479,10 +479,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>123</t>
-        </is>
+      <c r="A2" t="n">
+        <v>123</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -541,10 +539,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>123</t>
-        </is>
+      <c r="A3" t="n">
+        <v>123</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -601,6 +597,956 @@
           <t>linkedin.com/in/johndoe</t>
         </is>
       </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Immuno-Oncology Europe</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Immuno-Oncology</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Cookie Policy</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Immuno-Oncology Europe</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Immuno-Oncology</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Warning!</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Immuno-Oncology Europe</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Immuno-Oncology</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Filter by:</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Immuno-Oncology Europe</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Immuno-Oncology</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Abdelilah Aboussekhra</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Immuno-Oncology Europe</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Immuno-Oncology</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Abdelilah Aboussekhra</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Immuno-Oncology Europe</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Immuno-Oncology</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Balkese Alhamad</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Immuno-Oncology Europe</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Immuno-Oncology</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Balkese Alhamad</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Immuno-Oncology Europe</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Immuno-Oncology</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Andrew R Allen</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Immuno-Oncology Europe</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Immuno-Oncology</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Andrew R. Allen</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Immuno-Oncology Europe</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Immuno-Oncology</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Annarosa Arcangeli</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>CDX Europe</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Biomarkers &amp; Diagnostics</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Monika Lamba Saini</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>CDX Europe</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Biomarkers &amp; Diagnostics</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>EK Kim</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>CDX Europe</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Biomarkers &amp; Diagnostics</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Angela Douglas MBE</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>CDX Europe</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Biomarkers &amp; Diagnostics</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Nicole Chaves Petronzi</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>CDX Europe</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Biomarkers &amp; Diagnostics</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Catherine Mela</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>LNP Formulation</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Pharma Formulation</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Explore the 2026 Full Event Guide</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>LNP Formulation</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Pharma Formulation</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>LNP Characterization &amp; Analytical Development Summit</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>LNP Formulation</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Pharma Formulation</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Investigative &amp; Preclinical Toxicology Summit</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>LNP Formulation</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Pharma Formulation</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Extra-Hepatic Lipid-Based Nanoparticles Delivery Summit</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>LNP Formulation</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Pharma Formulation</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Lipid Nanoparticle Development Summit Europe</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Gene Therapy Conference</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Gene Therapy</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>What You Missed</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Gene Therapy Conference</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Gene Therapy</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Gene Therapy Analytical Development Summit</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Gene Therapy Conference</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Gene Therapy</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Viral Vectors Process Development &amp; Manufacturing Summit</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Gene Therapy Conference</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Gene Therapy</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Gene Therapy Analytical Development Summit Europe</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Gene Therapy Conference</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Gene Therapy</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Investigative &amp; Preclinical Toxicology Summit</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fixed the garbage data bug by using actual html selectors
</commit_message>
<xml_diff>
--- a/conference_data.xlsx
+++ b/conference_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -479,124 +479,104 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>123</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Pharma Test Conf</t>
+          <t>Peptide Summit</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Medicine</t>
+          <t>Peptides</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Oct 10-12, 2026</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>London, UK</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>John</t>
-        </is>
-      </c>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>John Doe</t>
+          <t>Tomi Sawyer</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Chief Scientist</t>
+          <t>Chief Drug Hunter &amp; President</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Big Pharma Inc</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>He does science</t>
-        </is>
-      </c>
+          <t>Maestro Therapeutics</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>URL here</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>linkedin.com/in/johndoe</t>
-        </is>
-      </c>
+          <t>https://peptide-based-therapeutics-summit.com/speaker/tomi-sawyer/</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>123</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Pharma Test Conf</t>
+          <t>Peptide Summit</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Medicine</t>
+          <t>Peptides</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Oct 10-12, 2026</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>London, UK</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>John</t>
-        </is>
-      </c>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>John Doe</t>
+          <t>Philip Jonas Sassene</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Chief Scientist</t>
+          <t>Scientific Director</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Big Pharma Inc</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>He does science</t>
-        </is>
-      </c>
+          <t>Novo Nordisk</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>URL here</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>linkedin.com/in/johndoe</t>
-        </is>
-      </c>
+          <t>https://peptide-based-therapeutics-summit.com/speaker/philip-jonas-sassene/</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -606,12 +586,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Immuno-Oncology Europe</t>
+          <t>Peptide Summit</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Immuno-Oncology</t>
+          <t>Peptides</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -627,13 +607,25 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Cookie Policy</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
+          <t>Cameron Pye</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Chief Executive Officer</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Unnatural Products</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>https://peptide-based-therapeutics-summit.com/speaker/cameron-pye/</t>
+        </is>
+      </c>
       <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
@@ -644,12 +636,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Immuno-Oncology Europe</t>
+          <t>Peptide Summit</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Immuno-Oncology</t>
+          <t>Peptides</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -665,13 +657,25 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Warning!</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
+          <t>Bradley Pentelute</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Associate Professor - Chemistry</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>https://peptide-based-therapeutics-summit.com/speaker/bradley-pentelute/</t>
+        </is>
+      </c>
       <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
@@ -682,12 +686,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Immuno-Oncology Europe</t>
+          <t>Peptide Summit</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Immuno-Oncology</t>
+          <t>Peptides</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -703,13 +707,25 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Filter by:</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
+          <t>Annette Bak</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Advanced Drug Delivery Head</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>AstraZeneca</t>
+        </is>
+      </c>
       <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>https://peptide-based-therapeutics-summit.com/speaker/annette-bak/</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr"/>
     </row>
     <row r="7">
@@ -720,12 +736,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Immuno-Oncology Europe</t>
+          <t>Peptide Summit</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Immuno-Oncology</t>
+          <t>Peptides</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -741,13 +757,25 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Abdelilah Aboussekhra</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
+          <t>Thomas Von Erlach</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Co-Founder &amp; Chief Scientific Officer</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Vivtex</t>
+        </is>
+      </c>
       <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>https://peptide-based-therapeutics-summit.com/speaker/thomas-von-erlach/</t>
+        </is>
+      </c>
       <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
@@ -758,12 +786,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Immuno-Oncology Europe</t>
+          <t>Peptide Summit</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Immuno-Oncology</t>
+          <t>Peptides</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -779,13 +807,25 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Abdelilah Aboussekhra</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
+          <t>Shelley Allen</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Project Director II, Peptide Discovery</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Abbvie</t>
+        </is>
+      </c>
       <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>https://peptide-based-therapeutics-summit.com/speaker/shelley-allen/</t>
+        </is>
+      </c>
       <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
@@ -796,12 +836,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Immuno-Oncology Europe</t>
+          <t>Peptide Summit</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Immuno-Oncology</t>
+          <t>Peptides</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -817,13 +857,25 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Balkese Alhamad</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
+          <t>Byungkook Lee</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Research &amp; Development Scientist</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Eli Lilly</t>
+        </is>
+      </c>
       <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>https://peptide-based-therapeutics-summit.com/speaker/byungkook-lee/</t>
+        </is>
+      </c>
       <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
@@ -834,12 +886,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Immuno-Oncology Europe</t>
+          <t>Peptide Summit</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Immuno-Oncology</t>
+          <t>Peptides</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -855,13 +907,25 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Balkese Alhamad</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
+          <t>Sumit Arora</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Senior Principal Scientist</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Johnson</t>
+        </is>
+      </c>
       <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>https://peptide-based-therapeutics-summit.com/speaker/sumit-arora/</t>
+        </is>
+      </c>
       <c r="L10" t="inlineStr"/>
     </row>
     <row r="11">
@@ -872,12 +936,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Immuno-Oncology Europe</t>
+          <t>Peptide Summit</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Immuno-Oncology</t>
+          <t>Peptides</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -893,13 +957,25 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Andrew R Allen</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
+          <t>Maria Fawaz</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Associate Principal Scientist, DMPK</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Merck &amp; Co</t>
+        </is>
+      </c>
       <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>https://peptide-based-therapeutics-summit.com/speaker/maria-fawaz/</t>
+        </is>
+      </c>
       <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
@@ -910,12 +986,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Immuno-Oncology Europe</t>
+          <t>CDX Europe</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Immuno-Oncology</t>
+          <t>Biomarkers &amp; Diagnostics</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -931,13 +1007,25 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Andrew R. Allen</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
+          <t>Monika Lamba Saini</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Director - Medical, Translational &amp; Computational Pathology</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>GSK</t>
+        </is>
+      </c>
       <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>https://cdx-europe.com/speaker/monika-lamba-saini/</t>
+        </is>
+      </c>
       <c r="L12" t="inlineStr"/>
     </row>
     <row r="13">
@@ -948,12 +1036,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Immuno-Oncology Europe</t>
+          <t>CDX Europe</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Immuno-Oncology</t>
+          <t>Biomarkers &amp; Diagnostics</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -969,13 +1057,25 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Annarosa Arcangeli</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
+          <t>EK Kim</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Head of Global Commercial Biomarkers &amp; Diagnostics</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Amgen</t>
+        </is>
+      </c>
       <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>https://cdx-europe.com/speaker/ek-kim/</t>
+        </is>
+      </c>
       <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
@@ -1007,13 +1107,25 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Monika Lamba Saini</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
+          <t>Angela Douglas MBE</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>President</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>British In Vitro Diagnostics Association</t>
+        </is>
+      </c>
       <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>https://cdx-europe.com/speaker/angela-douglas/</t>
+        </is>
+      </c>
       <c r="L14" t="inlineStr"/>
     </row>
     <row r="15">
@@ -1045,13 +1157,25 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>EK Kim</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
+          <t>Nicole Chaves Petronzi</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Senior Director, Global Regulatory Affairs Diagnostics</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Eli Lilly &amp; Co.</t>
+        </is>
+      </c>
       <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>https://cdx-europe.com/speaker/nicole-chaves-petronzi/</t>
+        </is>
+      </c>
       <c r="L15" t="inlineStr"/>
     </row>
     <row r="16">
@@ -1083,13 +1207,25 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Angela Douglas MBE</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
+          <t>Catherine Mela</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Head Precision Medicine Operations</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>GlaxoSmithKline</t>
+        </is>
+      </c>
       <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>https://cdx-europe.com/speaker/catherine-mela/</t>
+        </is>
+      </c>
       <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
@@ -1121,13 +1257,25 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Nicole Chaves Petronzi</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
+          <t>Jörg Engelbergs</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Scientific-Regulatory Assessor Targeted &amp; Personalized Biomedicines</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Paul-Ehrlich-Institut, National Competent Authority for Medicinal Products &amp; CDx Devices</t>
+        </is>
+      </c>
       <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>https://cdx-europe.com/speaker/jorg-engelbergs/</t>
+        </is>
+      </c>
       <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
@@ -1159,13 +1307,25 @@
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Catherine Mela</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
+          <t>Alastair Greystoke</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Honorary Medical Oncologist &amp; Professor of Oncology</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>The Newcastle upon Tyne Hospitals NHS Foundation Trust &amp; Newcastle University</t>
+        </is>
+      </c>
       <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>https://cdx-europe.com/speaker/alastair-greystoke/</t>
+        </is>
+      </c>
       <c r="L18" t="inlineStr"/>
     </row>
     <row r="19">
@@ -1176,12 +1336,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>LNP Formulation</t>
+          <t>CDX Europe</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Pharma Formulation</t>
+          <t>Biomarkers &amp; Diagnostics</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1197,13 +1357,25 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Explore the 2026 Full Event Guide</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
+          <t>Aino Telaranta-Keerie</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Senior Director, Global Precision Medicine Lead</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Astellas Pharma</t>
+        </is>
+      </c>
       <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>https://cdx-europe.com/speaker/aino-telaranta-keerie/</t>
+        </is>
+      </c>
       <c r="L19" t="inlineStr"/>
     </row>
     <row r="20">
@@ -1235,13 +1407,25 @@
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>LNP Characterization &amp; Analytical Development Summit</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
+          <t>Rushit Lodaya</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Associate Director - RNA Delivery Sciences</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>GlaxoSmithKline</t>
+        </is>
+      </c>
       <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>https://lnp-formulation-process-development-pharma.com/speaker/rushit-lodaya/</t>
+        </is>
+      </c>
       <c r="L20" t="inlineStr"/>
     </row>
     <row r="21">
@@ -1273,13 +1457,25 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Investigative &amp; Preclinical Toxicology Summit</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
+          <t>Michael Smith</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Senior Scientist - Drug Product Development</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Moderna</t>
+        </is>
+      </c>
       <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>https://lnp-formulation-process-development-pharma.com/speaker/michael-smith/</t>
+        </is>
+      </c>
       <c r="L21" t="inlineStr"/>
     </row>
     <row r="22">
@@ -1311,13 +1507,25 @@
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Extra-Hepatic Lipid-Based Nanoparticles Delivery Summit</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
+          <t>Emma Wang</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Chief Technology Officer</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>YolTech Therapeutics</t>
+        </is>
+      </c>
       <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>https://lnp-formulation-process-development-pharma.com/speaker/emma-wang/</t>
+        </is>
+      </c>
       <c r="L22" t="inlineStr"/>
     </row>
     <row r="23">
@@ -1349,13 +1557,25 @@
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Lipid Nanoparticle Development Summit Europe</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
+          <t>Gulen Tonga</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Principal Scientist</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Tessera Therapeutics</t>
+        </is>
+      </c>
       <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>https://lnp-formulation-process-development-pharma.com/speaker/gulen-tonga/</t>
+        </is>
+      </c>
       <c r="L23" t="inlineStr"/>
     </row>
     <row r="24">
@@ -1366,12 +1586,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Gene Therapy Conference</t>
+          <t>LNP Formulation</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Gene Therapy</t>
+          <t>Pharma Formulation</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1387,13 +1607,25 @@
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>What You Missed</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
+          <t>Ching Kim Tye</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Head of DP Platform and Early Clinical Development</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Sanofi</t>
+        </is>
+      </c>
       <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>https://lnp-formulation-process-development-pharma.com/speaker/ching-kim-tye/</t>
+        </is>
+      </c>
       <c r="L24" t="inlineStr"/>
     </row>
     <row r="25">
@@ -1404,12 +1636,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Gene Therapy Conference</t>
+          <t>LNP Formulation</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Gene Therapy</t>
+          <t>Pharma Formulation</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1425,13 +1657,25 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Gene Therapy Analytical Development Summit</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
+          <t>Annette Bak</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Executive Director</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>AstraZeneca</t>
+        </is>
+      </c>
       <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>https://lnp-formulation-process-development-pharma.com/speaker/annette-bak/</t>
+        </is>
+      </c>
       <c r="L25" t="inlineStr"/>
     </row>
     <row r="26">
@@ -1442,12 +1686,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Gene Therapy Conference</t>
+          <t>LNP Formulation</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Gene Therapy</t>
+          <t>Pharma Formulation</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1463,13 +1707,25 @@
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Viral Vectors Process Development &amp; Manufacturing Summit</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
+          <t>Luis Brito</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Vice President - Delivery Platform</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Beam Therapeutics</t>
+        </is>
+      </c>
       <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>https://lnp-formulation-process-development-pharma.com/speaker/luis-brito/</t>
+        </is>
+      </c>
       <c r="L26" t="inlineStr"/>
     </row>
     <row r="27">
@@ -1480,12 +1736,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Gene Therapy Conference</t>
+          <t>LNP Formulation</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Gene Therapy</t>
+          <t>Pharma Formulation</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1501,13 +1757,25 @@
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Gene Therapy Analytical Development Summit Europe</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
+          <t>Ching Kim Tye</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Head of DP Platform and Early Clinical Development</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Sanofi</t>
+        </is>
+      </c>
       <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>https://lnp-formulation-process-development-pharma.com/speaker/ching-kim-tye/</t>
+        </is>
+      </c>
       <c r="L27" t="inlineStr"/>
     </row>
     <row r="28">
@@ -1539,14 +1807,376 @@
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Investigative &amp; Preclinical Toxicology Summit</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
+          <t>Damir Simic</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Executive Director</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Astellas Pharma</t>
+        </is>
+      </c>
       <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>https://genetherapy-conference.com/speaker/damir-simic/</t>
+        </is>
+      </c>
       <c r="L28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Gene Therapy Conference</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Gene Therapy</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Jorge Santiago-Ortiz</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Senior Director - Chemistry, Manufacturing &amp; Controls</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Apertura Gene Therapy</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>https://genetherapy-conference.com/speaker/jorge-santiago-ortiz/</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Gene Therapy Conference</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Gene Therapy</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Devyn Smith</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Chief Executive Officer</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Arbor Biotechnologies, Inc.</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>https://genetherapy-conference.com/speaker/devyn-smith/</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Gene Therapy Conference</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Gene Therapy</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Hebe Sun</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Associate Director, CDx/IVD Regulatory Affairs</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Regeneron Pharmaceuticals</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>https://genetherapy-conference.com/speaker/hebe-sun/</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Gene Therapy Conference</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Gene Therapy</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Tassos Georgiadis</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Senior VP, Discovery &amp; Preclinical Development</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>MeiraGTx</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>https://genetherapy-conference.com/speaker/tassos-georgiadis/</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Gene Therapy Conference</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Gene Therapy</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Casey Maguire</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Investigator &amp; Associate Professor</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Harvard Medical School</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>https://genetherapy-conference.com/speaker/casey-maguire/</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Gene Therapy Conference</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Gene Therapy</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Lindsay Marjoram</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>CSO</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Barth Syndrome Foundation Inc</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>https://genetherapy-conference.com/speaker/lindsay-marjoram/</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Gene Therapy Conference</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Gene Therapy</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Susan serrano</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Senior Director, Market Access Strategy and Value Communication</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Intellia Therapeutics</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>https://genetherapy-conference.com/speaker/susan-serrano/</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
added speaker first name logic
</commit_message>
<xml_diff>
--- a/conference_data.xlsx
+++ b/conference_data.xlsx
@@ -504,7 +504,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Tomi</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr">
         <is>
           <t>Tomi Sawyer</t>
@@ -554,7 +558,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Philip</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr">
         <is>
           <t>Philip Jonas Sassene</t>
@@ -604,7 +612,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Cameron</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr">
         <is>
           <t>Cameron Pye</t>
@@ -654,7 +666,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Bradley</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr">
         <is>
           <t>Bradley Pentelute</t>
@@ -704,7 +720,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Annette</t>
+        </is>
+      </c>
       <c r="G6" t="inlineStr">
         <is>
           <t>Annette Bak</t>
@@ -754,7 +774,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Thomas</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr">
         <is>
           <t>Thomas Von Erlach</t>
@@ -804,7 +828,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Shelley</t>
+        </is>
+      </c>
       <c r="G8" t="inlineStr">
         <is>
           <t>Shelley Allen</t>
@@ -854,7 +882,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Byungkook</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr">
         <is>
           <t>Byungkook Lee</t>
@@ -904,7 +936,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Sumit</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr">
         <is>
           <t>Sumit Arora</t>
@@ -954,7 +990,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr">
         <is>
           <t>Maria Fawaz</t>
@@ -1004,7 +1044,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Monika</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr">
         <is>
           <t>Monika Lamba Saini</t>
@@ -1054,7 +1098,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>EK</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr">
         <is>
           <t>EK Kim</t>
@@ -1104,7 +1152,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Angela</t>
+        </is>
+      </c>
       <c r="G14" t="inlineStr">
         <is>
           <t>Angela Douglas MBE</t>
@@ -1154,7 +1206,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Nicole</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr">
         <is>
           <t>Nicole Chaves Petronzi</t>
@@ -1204,7 +1260,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Catherine</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr">
         <is>
           <t>Catherine Mela</t>
@@ -1254,7 +1314,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Jörg</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr">
         <is>
           <t>Jörg Engelbergs</t>
@@ -1304,7 +1368,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Alastair</t>
+        </is>
+      </c>
       <c r="G18" t="inlineStr">
         <is>
           <t>Alastair Greystoke</t>
@@ -1354,7 +1422,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Aino</t>
+        </is>
+      </c>
       <c r="G19" t="inlineStr">
         <is>
           <t>Aino Telaranta-Keerie</t>
@@ -1404,7 +1476,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Rushit</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr">
         <is>
           <t>Rushit Lodaya</t>
@@ -1454,7 +1530,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Michael</t>
+        </is>
+      </c>
       <c r="G21" t="inlineStr">
         <is>
           <t>Michael Smith</t>
@@ -1504,7 +1584,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Emma</t>
+        </is>
+      </c>
       <c r="G22" t="inlineStr">
         <is>
           <t>Emma Wang</t>
@@ -1554,7 +1638,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Gulen</t>
+        </is>
+      </c>
       <c r="G23" t="inlineStr">
         <is>
           <t>Gulen Tonga</t>
@@ -1604,7 +1692,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Ching</t>
+        </is>
+      </c>
       <c r="G24" t="inlineStr">
         <is>
           <t>Ching Kim Tye</t>
@@ -1654,7 +1746,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Annette</t>
+        </is>
+      </c>
       <c r="G25" t="inlineStr">
         <is>
           <t>Annette Bak</t>
@@ -1704,7 +1800,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Luis</t>
+        </is>
+      </c>
       <c r="G26" t="inlineStr">
         <is>
           <t>Luis Brito</t>
@@ -1754,7 +1854,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Ching</t>
+        </is>
+      </c>
       <c r="G27" t="inlineStr">
         <is>
           <t>Ching Kim Tye</t>
@@ -1804,7 +1908,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Damir</t>
+        </is>
+      </c>
       <c r="G28" t="inlineStr">
         <is>
           <t>Damir Simic</t>
@@ -1854,7 +1962,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
       <c r="G29" t="inlineStr">
         <is>
           <t>Jorge Santiago-Ortiz</t>
@@ -1904,7 +2016,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Devyn</t>
+        </is>
+      </c>
       <c r="G30" t="inlineStr">
         <is>
           <t>Devyn Smith</t>
@@ -1954,7 +2070,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Hebe</t>
+        </is>
+      </c>
       <c r="G31" t="inlineStr">
         <is>
           <t>Hebe Sun</t>
@@ -2004,7 +2124,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Tassos</t>
+        </is>
+      </c>
       <c r="G32" t="inlineStr">
         <is>
           <t>Tassos Georgiadis</t>
@@ -2054,7 +2178,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr"/>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Casey</t>
+        </is>
+      </c>
       <c r="G33" t="inlineStr">
         <is>
           <t>Casey Maguire</t>
@@ -2104,7 +2232,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Lindsay</t>
+        </is>
+      </c>
       <c r="G34" t="inlineStr">
         <is>
           <t>Lindsay Marjoram</t>
@@ -2154,7 +2286,11 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr"/>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Susan</t>
+        </is>
+      </c>
       <c r="G35" t="inlineStr">
         <is>
           <t>Susan serrano</t>

</xml_diff>

<commit_message>
implemented deep scraping for speaker profiles and photo downloads
</commit_message>
<xml_diff>
--- a/conference_data.xlsx
+++ b/conference_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:N34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,6 +474,16 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
+          <t>Speaker Image URL</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Speaker Image Local Path</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
           <t>Speaker LinkedIn</t>
         </is>
       </c>
@@ -481,7 +491,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-920281</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -524,18 +534,39 @@
           <t>Maestro Therapeutics</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Thank you to our speakers, sponsors, and delegates who joined us in Boston for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
+Tomi is an entrepreneurial drug hunter with &gt;40 years of industrial experience in both large pharma and biotech. He has three marketed drugs and &gt;670 scientific publications, patents, and presentations (primarily focused on peptide drug discovery). Tomi is the Founding President of the Peptide Drug Hunting Consortium.
+This your chance to hear from pioneering executive leaders the peptide space who will discuss their ambitions, strategies and challenges for peptide discovery, targets. indications and development of next generation of peptide drugs.
+We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
+Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
+This website uses the following types of services. Learn more from our
+                    Cookie Policy.
+By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+        </is>
+      </c>
       <c r="K2" t="inlineStr">
         <is>
           <t>https://peptide-based-therapeutics-summit.com/speaker/tomi-sawyer/</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>https://peptide-based-therapeutics-summit.com/wp-content/uploads/sites/255/2025/11/Tomi-Sawyer-300x300.png</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>images/tomi_sawyer.jpg</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-920281</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -578,18 +609,38 @@
           <t>Novo Nordisk</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Thank you to our speakers, sponsors, and delegates who joined us in Boston for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
+Philip Jonas Sassene has a strong track record in drug delivery. He has 15+ years of experience in enabling formulations with particular emphasis on enabling formulation strategies for oral delivery of peptides &amp; proteins. He is currently employed as a Scientific Director within oral delivery technologies at Novo Nordisk A/S.
+We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
+Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
+This website uses the following types of services. Learn more from our
+                    Cookie Policy.
+By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+        </is>
+      </c>
       <c r="K3" t="inlineStr">
         <is>
           <t>https://peptide-based-therapeutics-summit.com/speaker/philip-jonas-sassene/</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>https://peptide-based-therapeutics-summit.com/wp-content/uploads/sites/255/2025/12/Philip-Sassene-300x300.png</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>images/philip_jonas_sassene.jpg</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-920281</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -632,18 +683,38 @@
           <t>Unnatural Products</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Thank you to our speakers, sponsors, and delegates who joined us in Boston for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
+The biopharmaceutical sector continues to innovate peptide discovery innovations, from new macrocycles to new delivery methods and are thriving on strategic alliances, which allow for cross-functional sharing of knowledge, and experience to advance peptide drugs to patients faster. Hear first-hand how investors and key biotechs are keeping up with the peptide momentum through investments, alliances and collaborations.
+We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
+Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
+This website uses the following types of services. Learn more from our
+                    Cookie Policy.
+By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+        </is>
+      </c>
       <c r="K4" t="inlineStr">
         <is>
           <t>https://peptide-based-therapeutics-summit.com/speaker/cameron-pye/</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>https://peptide-based-therapeutics-summit.com/wp-content/uploads/sites/255/2025/11/Cameron-P-300x300.png</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>images/cameron_pye.jpg</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-920281</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -686,18 +757,38 @@
           <t>MIT</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Thank you to our speakers, sponsors, and delegates who joined us in Boston for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
+Bradley L. Pentelute is a Professor of Chemistry at MIT (https://pentelutelabmit.com). He is also an Associate Member, Broad Institute of Harvard and MIT, an Extramural Member of the MIT Koch Cancer Institute, and Member, Center for Environmental Health Sciences MIT. He received his undergraduate degree in Psychology and Chemistry from the University of Southern California, and his M.S and Ph.D. in Organic Chemistry from the University of Chicago with Prof. Steve Kent. He was a postdoctoral fellow in the laboratory of Dr. R. John Collier at Harvard Medical School, Microbiology.
+We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
+Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
+This website uses the following types of services. Learn more from our
+                    Cookie Policy.
+By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+        </is>
+      </c>
       <c r="K5" t="inlineStr">
         <is>
           <t>https://peptide-based-therapeutics-summit.com/speaker/bradley-pentelute/</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>https://peptide-based-therapeutics-summit.com/wp-content/uploads/sites/255/2025/11/Bradley-P-300x300.png</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>images/bradley_pentelute.jpg</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-920281</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -740,18 +831,42 @@
           <t>AstraZeneca</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Thank you to our speakers, sponsors, and delegates who joined us in Boston for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
+Annette Bak, Ph.D., MBA, leads Advanced Drug Delivery (ADD) at AstraZeneca and serves on the Pharmaceutical Sciences leadership team. ADD, a global organization with over 100 employees in Sweden, UK, and US, aims to transform diverse modalities into investigational medicines.
+Since joining AstraZeneca in 2016, Annette has delivered various synthetic modalities and mRNA drug delivery systems for preclinical and clinical studies. She has also built delivery chemistry, intracellular drug delivery capabilities, and a search and evaluation group within ADD.
+Previously, Annette worked for Amgen and Merck in the US, focusing on small molecule and peptide formulations, outsourcing partnerships in China, and in-licensing and partnership evaluations. She contributed to bringing small molecule therapies to market.
+Annette has published over 50 articles, given more than 50 invited presentations, and serves on the editorial boards of the Journal of Pharmaceutical Sciences and Molecular Pharmaceutics. She holds several patents for pharmaceutical technologies.
+A key volunteer in the American Association of Pharmaceutical Scientists (AAPS), Annette was the 2022 president, leading the implementation of the 2021-2025 strategic plan. She was the 2020 co-recipient of the AAPS Alice E. Till Women in Pharmaceutical Science Recognition.
+We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
+Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
+This website uses the following types of services. Learn more from our
+                    Cookie Policy.
+By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+        </is>
+      </c>
       <c r="K6" t="inlineStr">
         <is>
           <t>https://peptide-based-therapeutics-summit.com/speaker/annette-bak/</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>https://peptide-based-therapeutics-summit.com/wp-content/uploads/sites/255/2025/11/Annette-B-300x300.png</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>images/annette_bak.jpg</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-920281</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -794,18 +909,39 @@
           <t>Vivtex</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Thank you to our speakers, sponsors, and delegates who joined us in Boston for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
+Thomas von Erlach, PhD co-founded Vivtex and joined as its Chief Scientific Officer when Vivtex was formed as a MIT spin-off in 2018. Prior to that he led the interdisciplinary efforts around gastrointestinal model systems for oral drug delivery applications at the Laboratory of Prof. Robert Langer and Prof. Giovanni Traverso at MIT. Dr von Erlach obtained his PhD from Imperial College London in Bioengineering and a BSc and MSc in Biochemistry and Biotechnology from ETH Zurich in Switzerland. His research interest include advanced in vitro models for drug development, oral drug delivery and gastrointestinal pharmacology. His work is published in several high impact journals such as Nature Materials, Nature Biomedical Engineering, and Nature Communications.
+The biopharmaceutical sector continues to innovate peptide discovery innovations, from new macrocycles to new delivery methods and are thriving on strategic alliances, which allow for cross-functional sharing of knowledge, and experience to advance peptide drugs to patients faster. Hear first-hand how investors and key biotechs are keeping up with the peptide momentum through investments, alliances and collaborations.
+We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
+Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
+This website uses the following types of services. Learn more from our
+                    Cookie Policy.
+By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+        </is>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>https://peptide-based-therapeutics-summit.com/speaker/thomas-von-erlach/</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>https://peptide-based-therapeutics-summit.com/wp-content/uploads/sites/255/2025/11/Thomas-V-300x300.png</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>images/thomas_von_erlach.jpg</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-920281</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -848,18 +984,40 @@
           <t>Abbvie</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Thank you to our speakers, sponsors, and delegates who joined us in Boston for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
+Shelley Allen is an accomplished drug discovery leader with more than 25 years of experience in medicinal chemistry. She has a proven history of building and leading successful teams in both biotech and pharma, consistently delivering high-quality drug candidates with a strong sense of urgency. Shelley served as the Head of Drug Discovery at Nimble Therapeutics until its acquisition by AbbVie earlier this year. She now continues her impactful work at AbbVie, contributing to the discovery and development of peptide programs within the Immuno-Pharmacology &amp; Peptide Discovery group.
+Practical Approaches to Characterize ADME &amp; Design Translatable In Vitro &amp; In Vivo PK/PD Studies with Jianzhong Wen
+Improving Permeating Agent Performance to Achieve Successful Peptide Oral Bioavailability with Shelley Allen
+We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
+Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
+This website uses the following types of services. Learn more from our
+                    Cookie Policy.
+By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+        </is>
+      </c>
       <c r="K8" t="inlineStr">
         <is>
           <t>https://peptide-based-therapeutics-summit.com/speaker/shelley-allen/</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>https://peptide-based-therapeutics-summit.com/wp-content/uploads/sites/255/2025/11/Shelley-A-1-300x300.png</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>images/shelley_allen.jpg</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-920281</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -902,18 +1060,38 @@
           <t>Eli Lilly</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Thank you to our speakers, sponsors, and delegates who joined us in Boston for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
+Qook Lee joined the BioTDR group at Eli Lilly as a Research Scientist in 2017 and currently serves as a Research Advisor (Engineer) in Lilly Genetic Medicine at the Lilly Seaport Innovation Center. His work has focused on developing oral GG and GGG delivery platforms using hydrogels, polymeric particles, minitablets, and other technologies for extended drug delivery platform. He has also contributed to the evaluation of formulation and analytical method development in the mRNA-LNP-based protein replacement therapeutic area, gene editing and LNP production process development and supported large animal study productions.
+We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
+Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
+This website uses the following types of services. Learn more from our
+                    Cookie Policy.
+By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+        </is>
+      </c>
       <c r="K9" t="inlineStr">
         <is>
           <t>https://peptide-based-therapeutics-summit.com/speaker/byungkook-lee/</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>https://peptide-based-therapeutics-summit.com/wp-content/uploads/sites/255/2025/11/Qook-Lee-300x300.png</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>images/byungkook_lee.jpg</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-920281</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -956,18 +1134,37 @@
           <t>Johnson &amp; Johnson</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Thank you to our speakers, sponsors, and delegates who joined us in Boston for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
+We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
+Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
+This website uses the following types of services. Learn more from our
+                    Cookie Policy.
+By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+        </is>
+      </c>
       <c r="K10" t="inlineStr">
         <is>
           <t>https://peptide-based-therapeutics-summit.com/speaker/sumit-arora/</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>https://peptide-based-therapeutics-summit.com/wp-content/uploads/sites/255/2025/11/Sumit-Arora-300x300.png</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>images/sumit_arora.jpg</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-920281</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1010,18 +1207,38 @@
           <t>Merck &amp; Co</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Thank you to our speakers, sponsors, and delegates who joined us in Boston for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
+Dr. Maria Fawaz is an Associate Principal Scientist in Pharmacokinetics, Dynamics, Metabolism &amp; Bioanalytics at Merck Research Laboratories, West Point, PA. As a DMPK principal investigator, Maria supports various peptide modalities, guiding design strategies in the early discovery space, lead optimization, and also supports clinical-stage programs. Maria has extensive experience in cyclic peptide metabolite identification, where she co-discovered novel analytical strategies of unambiguously identifying regions in the cyclic peptide sequence susceptible to amide hydrolysis by proteases. At Merck, Maria is also working with external collaborators and various funding organizations. Maria holds a PhD degree in Medicinal Chemistry from the University of Michigan. Her doctoral research was focused on the design and synthesis of high-density lipoproteins (sHDL) composed of ApoA-I mimetic peptides and phospholipids for the treatment of Niemann-Pick diseases and atherosclerosis. Maria is passionate about mentoring junior scientists and she is actively engaged in student and postdoc career outreach at various universities.
+We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
+Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
+This website uses the following types of services. Learn more from our
+                    Cookie Policy.
+By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+        </is>
+      </c>
       <c r="K11" t="inlineStr">
         <is>
           <t>https://peptide-based-therapeutics-summit.com/speaker/maria-fawaz/</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>https://peptide-based-therapeutics-summit.com/wp-content/uploads/sites/255/2025/11/Maria-F-300x300.png</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>images/maria_fawaz.jpg</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-5F4D69</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1064,18 +1281,44 @@
           <t>GSK</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Why Not Join Us for the Next Event in the World Biomarkers &amp; Diagnostics Series?
+Discover the 16th World Clinical Biomarkers &amp; CDx Summit here
+Thank you to our speakers, sponsors, and delegates who joined us in London for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
+Why Not Join Us for the Next Event in the World Biomarkers &amp; Diagnostics Series?
+Discover the 16th World Clinical Biomarkers &amp; CDx Summit here
+Thank you to our speakers, sponsors, and delegates who joined us in London for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
+Director - Medical, Translational &amp; Computational Pathology GSK
+Monika Lamba Saini is a highly skilled professional currently serving as the Global Translational Pathology Leader at ADC Therapeutics since August 2024, where strategic leadership is provided to enhance the understanding of diseases and to implement translational research strategies for developing novel therapeutics. In addition, Monika is an Education Committee Member at the Digital Pathology Association, contributing to webinars and academic content. Prior experience includes roles as Director of Digital Pathology Innovation and Pathology Research Scientist at IQVIA Laboratories, focusing on digital pathology and AI-driven trials, and as a Pathologist and Principal Investigator at CellCarta, specializing in histopathological evaluations of cancers and immune-oncology therapies. Monika also has an extensive academic background, including a PhD in Biomedical Sciences and a Doctor of Medicine degree in Pathology from esteemed institutions.
+We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
+Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
+This website uses the following types of services. Learn more from our
+                    Cookie Policy.
+By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+        </is>
+      </c>
       <c r="K12" t="inlineStr">
         <is>
           <t>https://cdx-europe.com/speaker/monika-lamba-saini/</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>https://cdx-europe.com/wp-content/uploads/sites/254/2025/12/monika-Lamba-Saini-300x300.png</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>images/monika_lamba_saini.jpg</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-5F4D69</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1118,18 +1361,44 @@
           <t>Amgen</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Why Not Join Us for the Next Event in the World Biomarkers &amp; Diagnostics Series?
+Discover the 16th World Clinical Biomarkers &amp; CDx Summit here
+Thank you to our speakers, sponsors, and delegates who joined us in London for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
+Why Not Join Us for the Next Event in the World Biomarkers &amp; Diagnostics Series?
+Discover the 16th World Clinical Biomarkers &amp; CDx Summit here
+Thank you to our speakers, sponsors, and delegates who joined us in London for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
+Head of Global Commercial Biomarkers &amp; Diagnostics Amgen
+EK Kim is the Global Head of Commercial Biomarkers and Diagnostics at Amgen, where she leads the commercialization and launch strategy for diagnostic and patient identification tools across oncology, cardiovascular, inflammation, and rare disease. She has held leadership roles across commercial and development functions and has directed global readiness for multiple integrated medicine and diagnostic launches. Prior to Amgen, EK held senior roles at AstraZeneca, Personal Genome Diagnostics (PGDx), Roche Diagnostics, and Ventana Medical Systems, where she advanced precision medicine strategies that supported global brand planning, development and regulatory planning, and commercialization.
+We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
+Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
+This website uses the following types of services. Learn more from our
+                    Cookie Policy.
+By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+        </is>
+      </c>
       <c r="K13" t="inlineStr">
         <is>
           <t>https://cdx-europe.com/speaker/ek-kim/</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>https://cdx-europe.com/wp-content/uploads/sites/254/2025/12/EK-Kim-300x300.png</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>images/ek_kim.jpg</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-5F4D69</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1172,18 +1441,49 @@
           <t>British In Vitro Diagnostics Association</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Why Not Join Us for the Next Event in the World Biomarkers &amp; Diagnostics Series?
+Discover the 16th World Clinical Biomarkers &amp; CDx Summit here
+Thank you to our speakers, sponsors, and delegates who joined us in London for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
+Why Not Join Us for the Next Event in the World Biomarkers &amp; Diagnostics Series?
+Discover the 16th World Clinical Biomarkers &amp; CDx Summit here
+Thank you to our speakers, sponsors, and delegates who joined us in London for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
+Angela is an Inspirational leader with a demonstrated history of working previously in the NHS for over 42 years, as DCSO and in Genetics and Genomics, as the Scientific Director of a Regional Genomics Service and Clinical Programme Director of the NW Coast Genomic Medicine Centre.
+She retired from the post of the Deputy Chief Scientific Officer (DCSO) for NHS England in October 2023, after holding the position for 5 yrs. Angela is now the President of BIVDA having taken up this role in December 2023. She is an influential, collaborative team leader with a proven record in Clinical Research, Medical Education, Mentoring and Coaching, in Life Sciences.
+Angela has a strong financial acumen and is a strategic leadership expert. She is passionate about quality assurance, safety and regulation in Science and in particular Genetics and Genomics, her area of expertise. She graduated from University College London and is a Fellow of the Royal College of Pathologists and an honorary Fellow of the Academy for Healthcare Science.
+She had the pleasure of being the President of the BSGM, Chairman of the RCPath Genetics and Reproductive Medicines Specialist Advisory Committee and was RCPath’s Scientific Lead before taking on the role of DCSO.
+In 2014, Angela was named as one of HSJ’s top 50 Inspirational Women. In 2015, she was awarded NHS Healthcare Scientist of the Year, and in 2016, was honoured in Her Majesty the Queen’s 90th Birthday Honours List as a Member of the Order of the British Empire for Research and Mentoring Students.
+In 2019, she was included in the Pathologist Power list as one of the top 100 trailblazers. In 2021, Angela was delighted to be approved as an Honorary Fellow of IPEM. In 2022 her leadership journey was published in Snapshots of Women in COG. In 2023, the AHCS again recognised her contribution to education and training with a second Fellowship.
+In 2023, Angela was nominated as a Woman of the Year by the Women Leaders Network. Angela is an inclusive, compassionate and kind leader with a broad experience of working across the healthcare system, and in all her endeavours strives to bring out the best in all those she works with.
+We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
+Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
+This website uses the following types of services. Learn more from our
+                    Cookie Policy.
+By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+        </is>
+      </c>
       <c r="K14" t="inlineStr">
         <is>
           <t>https://cdx-europe.com/speaker/angela-douglas/</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr"/>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>https://cdx-europe.com/wp-content/uploads/sites/254/2025/12/Angela-Douglas-300x300.png</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>images/angela_douglas_mbe.jpg</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-5F4D69</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1226,18 +1526,44 @@
           <t>Eli Lilly &amp; Co.</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Why Not Join Us for the Next Event in the World Biomarkers &amp; Diagnostics Series?
+Discover the 16th World Clinical Biomarkers &amp; CDx Summit here
+Thank you to our speakers, sponsors, and delegates who joined us in London for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
+Why Not Join Us for the Next Event in the World Biomarkers &amp; Diagnostics Series?
+Discover the 16th World Clinical Biomarkers &amp; CDx Summit here
+Thank you to our speakers, sponsors, and delegates who joined us in London for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
+Senior Director, Global Regulatory Affairs Diagnostics Eli Lilly &amp; Co.
+Nicole Chaves Petronzi is Senior Director of Global Regulatory Affairs Diagnostics at Lilly. With extensive experience in in-vitro diagnostics and pharmaceutical regulatory strategy, Nicole has led global initiatives to implement the EU IVDR and harmonize compliance across multiple markets. Her work focuses on integrating diagnostics into pharmaceutical development, driving collaboration between Regulatory Affairs, Quality, Clinical, and Laboratory teams to accelerate innovation and patient access. Nicole is recognized for her ability to navigate complex regulatory landscapes and transform compliance into a strategic advantage for diagnostics in pharma.
+We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
+Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
+This website uses the following types of services. Learn more from our
+                    Cookie Policy.
+By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+        </is>
+      </c>
       <c r="K15" t="inlineStr">
         <is>
           <t>https://cdx-europe.com/speaker/nicole-chaves-petronzi/</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr"/>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>https://cdx-europe.com/wp-content/uploads/sites/254/2025/12/Nicole-Chaves-Petronzi-300x300.png</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>images/nicole_chaves_petronzi.jpg</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-5F4D69</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1280,18 +1606,45 @@
           <t>GlaxoSmithKline</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Why Not Join Us for the Next Event in the World Biomarkers &amp; Diagnostics Series?
+Discover the 16th World Clinical Biomarkers &amp; CDx Summit here
+Thank you to our speakers, sponsors, and delegates who joined us in London for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
+Why Not Join Us for the Next Event in the World Biomarkers &amp; Diagnostics Series?
+Discover the 16th World Clinical Biomarkers &amp; CDx Summit here
+Thank you to our speakers, sponsors, and delegates who joined us in London for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
+Dr Catherine Mela is Head of Biomarker Operations, within GSK. In her role, Catherine is accountable for leading the Scientific Operations and Data Operations teams, driving the execution of precision medicine project strategies with efficiency and quality.
+Catherine has gained broad experience in laboratory and bio-sample operations, while leading Human Biological Sample operational and governance teams in AstraZeneca and Roche.
+Prior to working in pharma, Catherine’s background was in Clinical research within the NHS. She holds a PhD from Imperial College on ‘The impact of treatment strategies on immune responses in HIV-1 infection’. Catherine is a fellow of the institute of leadership and is passionate about professional development, mentorship and creating a supportive environment for individuals within her teams.
+We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
+Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
+This website uses the following types of services. Learn more from our
+                    Cookie Policy.
+By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+        </is>
+      </c>
       <c r="K16" t="inlineStr">
         <is>
           <t>https://cdx-europe.com/speaker/catherine-mela/</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr"/>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>https://cdx-europe.com/wp-content/uploads/sites/254/2025/12/Catherine-Mela-300x300.png</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>images/catherine_mela.jpg</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-5F4D69</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1334,18 +1687,45 @@
           <t>Paul-Ehrlich-Institut, National Competent Authority for Medicinal Products &amp; CDx Devices</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Why Not Join Us for the Next Event in the World Biomarkers &amp; Diagnostics Series?
+Discover the 16th World Clinical Biomarkers &amp; CDx Summit here
+Thank you to our speakers, sponsors, and delegates who joined us in London for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
+Why Not Join Us for the Next Event in the World Biomarkers &amp; Diagnostics Series?
+Discover the 16th World Clinical Biomarkers &amp; CDx Summit here
+Thank you to our speakers, sponsors, and delegates who joined us in London for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
+Scientific-Regulatory Assessor Targeted &amp; Personalized Biomedicines Paul-Ehrlich-Institut, National Competent Authority for Medicinal Products &amp; CDx Devices
+Jörg Engelbergs is currently working for the Paul-Ehrlich-Institut (PEI), German National Competent Authority for Medicinal Products and CDx devices, as a scientific-regulatory assessor (Quality, Non-Clinic, Biomarkers, CDx). He is involved in the European process of marketing authorization and life cycle of predictive biomarker guided biopharmaceuticals comprising scientific assessments and advices. Further tasks are assessments of CTR conformity of clinical trials and IVDR conformity of associated CDx performance studies. He is also responsible for the technical, procedural and scientific implementation of the new responsibility of PEI for CDx performance studies. At the European level he is member of several CDx related European working groups, e.g. EMA CHMP/CAT CDx Expert Group (Co-Chair), EMA Methodology Working Party, EMA SIA PGx (Leadership Team), and EU COMBINE Project.
+He holds a Diploma in biology and a PhD. He has extensive experience as scientific project leader in cancer research at the West German Cancer Center (WTZE) and in neuropharmacology research, including R&amp;D of diagnostic/predictive biomarkers and assays, as well as in the establishment and management of a central clinical genotyping service center at the Medical Faculty of the University of Essen, Germany.
+We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
+Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
+This website uses the following types of services. Learn more from our
+                    Cookie Policy.
+By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+        </is>
+      </c>
       <c r="K17" t="inlineStr">
         <is>
           <t>https://cdx-europe.com/speaker/jorg-engelbergs/</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr"/>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>https://cdx-europe.com/wp-content/uploads/sites/254/2025/12/Jorg-Engelbergs-300x300.png</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>images/jörg_engelbergs.jpg</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-5F4D69</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1388,18 +1768,44 @@
           <t>The Newcastle upon Tyne Hospitals NHS Foundation Trust &amp; Newcastle University</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Why Not Join Us for the Next Event in the World Biomarkers &amp; Diagnostics Series?
+Discover the 16th World Clinical Biomarkers &amp; CDx Summit here
+Thank you to our speakers, sponsors, and delegates who joined us in London for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
+Why Not Join Us for the Next Event in the World Biomarkers &amp; Diagnostics Series?
+Discover the 16th World Clinical Biomarkers &amp; CDx Summit here
+Thank you to our speakers, sponsors, and delegates who joined us in London for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
+Honorary Medical Oncologist &amp; Professor of Oncology The Newcastle upon Tyne Hospitals NHS Foundation Trust &amp; Newcastle University
+Professor Greystoke joined Newcastle University and the Northern Centre for Cancer Care in 2014 after 8 years spent at the University of Manchester/ Christie NHS Trust. He is one of 4 consultants that run the Sir Bobby Robson Early Clinical Trials Centre at the Freeman hospital in Newcastle,and has a special interest in the development of new anti-cancer drugs for patients with lung cancer. He leads systemic therapy research for NSCLC in the North-East, with a portfolio of Phase I-IV studies. In addition he is the Clinical Director for Cancer for the Yorkshire, Hull and North East England Genomic Medicine Service and led the NHSE pilot assessing the cost-effectiveness of cfDNA in patients presenting with advanced lung cancer. He is the Joint Chief Investigator of the CONCORDE platform (adding in new drugs to radical radiotherapy in lung cancer), and leads the Pharmacodynamic Biomarker team at Newcastle University Cancer.
+We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
+Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
+This website uses the following types of services. Learn more from our
+                    Cookie Policy.
+By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+        </is>
+      </c>
       <c r="K18" t="inlineStr">
         <is>
           <t>https://cdx-europe.com/speaker/alastair-greystoke/</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr"/>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>https://cdx-europe.com/wp-content/uploads/sites/254/2025/12/Alastair-Greystoke-300x300.png</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>images/alastair_greystoke.jpg</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-5F4D69</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1442,18 +1848,44 @@
           <t>Astellas Pharma</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Why Not Join Us for the Next Event in the World Biomarkers &amp; Diagnostics Series?
+Discover the 16th World Clinical Biomarkers &amp; CDx Summit here
+Thank you to our speakers, sponsors, and delegates who joined us in London for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
+Why Not Join Us for the Next Event in the World Biomarkers &amp; Diagnostics Series?
+Discover the 16th World Clinical Biomarkers &amp; CDx Summit here
+Thank you to our speakers, sponsors, and delegates who joined us in London for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
+Senior Director, Global Precision Medicine Lead Astellas Pharma
+Aino Telaranta-Keerie has worked 20+ years in the pharmaceutical and diagnostic industries, with 10+ years’ experience as Precision Medicine leader in oncology at AstraZeneca and Astellas. She is passionate about optimising CDx partnerships and strategies to ensure successful development of new therapies for patients.
+We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
+Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
+This website uses the following types of services. Learn more from our
+                    Cookie Policy.
+By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+        </is>
+      </c>
       <c r="K19" t="inlineStr">
         <is>
           <t>https://cdx-europe.com/speaker/aino-telaranta-keerie/</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr"/>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>https://cdx-europe.com/wp-content/uploads/sites/254/2025/12/Aino-Telaranta-Keerie-300x300.png</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>images/aino_telarantakeerie.jpg</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-282EB2</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1496,18 +1928,39 @@
           <t>GlaxoSmithKline</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr"/>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Associate Director - RNA Delivery Sciences GlaxoSmithKline
+Dr. Rushit Lodaya is Associate Director and RNA Delivery Lead at GSK’s RNA Center of Excellence, where he advances delivery platforms for vaccines and infectious diseases. He specializes in Lipid Nanoparticle (LNP) formulation, scale-up process optimization, and the thermostability of multicomponent systems, including mRNA-LNPs. His expertise also extends to vaccine adjuvant formulation and the optimization of novel adjuvants to enhance immune responses. Dr. Lodaya earned his PhD at Northeastern University under the mentorship of Dr. Mansoor Amiji and Dr. Derek O’Hagan, where he developed a strong foundation in nanomedicine and translational vaccine research.
+With immune responses, from anti-PEG and ligand antibodies to component-linked immunogenicity, impacting LNP dosing regimens and limiting clinical success. This workshop will delve into advanced analytics for understanding safety and evaluate innovative solutions to achieve effective repeat dosing.
+We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
+Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
+This website uses the following types of services. Learn more from our
+                    Cookie Policy.
+By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+        </is>
+      </c>
       <c r="K20" t="inlineStr">
         <is>
           <t>https://lnp-formulation-process-development-pharma.com/speaker/rushit-lodaya/</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr"/>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>https://lnp-formulation-process-development-pharma.com/wp-content/uploads/sites/241/2025/11/Rushit-Lodaya-300x300.png</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>images/rushit_lodaya.jpg</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-282EB2</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1550,18 +2003,39 @@
           <t>Moderna</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Senior Scientist - Drug Product Development Moderna
+Michael “Mike” Smith currently serves as Director of the Emerging Technologies group at Moderna. In his role, Mike leads a cross-disciplinary science and engineering team developing lipid nanoparticle (LNP) formulation platforms for messenger RNA (mRNA). Mike is a self-proclaimed “nanoparticle geek” and has a deep curiosity for the physical chemistry of nanoparticle self-assembly. Leveraging the science of nanoparticle synthesis, the team has built robust scale-up capabilities that service Moderna’s ambitious development portfolio, which includes over 40 drug candidates in active development. Mike and team were major contributors towards the development of Moderna vaccine against SARS-COVID-2 (mRNA-1273). His efforts, together with the Moderna team, were featured in a CNN Hero’s segment and further showcased in NY Magazine (see links below).
+Mike has led numerous scientific and engineering projects over eleven years at Moderna. In years prior, Mike contributed to nanoparticle formulation efforts at Merck that include siRNA LNP and liposomal formulations. Prior to his time in industry, Mike received his PhD from Georgia Tech with a dissertation on the topic of stimuli-responsive hydrogel nanoparticles for therapeutic delivery.
+We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
+Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
+This website uses the following types of services. Learn more from our
+                    Cookie Policy.
+By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+        </is>
+      </c>
       <c r="K21" t="inlineStr">
         <is>
           <t>https://lnp-formulation-process-development-pharma.com/speaker/michael-smith/</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr"/>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>https://lnp-formulation-process-development-pharma.com/wp-content/uploads/sites/241/2025/11/Michael-Smith-300x300.png</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>images/michael_smith.jpg</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-282EB2</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1604,18 +2078,37 @@
           <t>YolTech Therapeutics</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr"/>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Dr. Emma Wang is the chief technology officer and co-founder at YolTech Therapeutics. Her focus is on advancing the non-viral delivery platform to support in vivo gene therapy development through research in novel lipid discovery, product development, process development, characterization as well as GMP manufacture. Prior to joining YolTech, Emma held research positions of growing responsibilities at Providence Therapeutics and Beam Therapeutics. Emma holds a Ph.D. in Chemistry as a member of Prof. Katharina Landfester’s group from Max Planck Institute for Polymer Research in Germany, a M.Eng and B.Eng in Chemical Engineering from McGill University in Canada.
+We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
+Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
+This website uses the following types of services. Learn more from our
+                    Cookie Policy.
+By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+        </is>
+      </c>
       <c r="K22" t="inlineStr">
         <is>
           <t>https://lnp-formulation-process-development-pharma.com/speaker/emma-wang/</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr"/>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>https://lnp-formulation-process-development-pharma.com/wp-content/uploads/sites/241/2025/11/Emma-Wang-300x300.png</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>images/emma_wang.jpg</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-282EB2</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1658,18 +2151,36 @@
           <t>Tessera Therapeutics</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
+Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
+This website uses the following types of services. Learn more from our
+                    Cookie Policy.
+By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+        </is>
+      </c>
       <c r="K23" t="inlineStr">
         <is>
           <t>https://lnp-formulation-process-development-pharma.com/speaker/gulen-tonga/</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr"/>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>https://lnp-formulation-process-development-pharma.com/wp-content/uploads/sites/241/2026/02/Gulen-Tonga-300x300.png</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>images/gulen_tonga.jpg</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-282EB2</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1712,18 +2223,39 @@
           <t>Sanofi</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Head of DP Platform and Early Clinical Development Sanofi
+Dr. Ching Kim Tye brings two decades of pharmaceutical R&amp;D expertise, specializing in formulation and drug delivery systems. As Head of Drug Product Platform and Early Clinical Development at Sanofi, she leads innovation in mRNA-LNP technology development.
+Currently, Kim spearheads the development of next-generation LNPs with enhanced potency and thermostability for both intramuscular and intranasal delivery routes, advancing candidates into Phase 1 clinical trials. Her comprehensive experience spans from early research through late-stage development, including work with diverse therapeutic modalities—proteins and small molecules at CSL, Pfizer, and Eli Lilly.
+We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
+Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
+This website uses the following types of services. Learn more from our
+                    Cookie Policy.
+By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+        </is>
+      </c>
       <c r="K24" t="inlineStr">
         <is>
           <t>https://lnp-formulation-process-development-pharma.com/speaker/ching-kim-tye/</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr"/>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>https://lnp-formulation-process-development-pharma.com/wp-content/uploads/sites/241/2025/11/Ching-Kim-Tye-300x300.png</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>images/ching_kim_tye.jpg</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-282EB2</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1766,18 +2298,41 @@
           <t>AstraZeneca</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Annette Bak, Ph.D., MBA, leads Advanced Drug Delivery (ADD) at AstraZeneca and serves on the Pharmaceutical Sciences leadership team. ADD, a global organization with over 100 employees in Sweden, UK, and US, aims to transform diverse modalities into investigational medicines.
+Since joining AstraZeneca in 2016, Annette has delivered various synthetic modalities and mRNA drug delivery systems for preclinical and clinical studies. She has also built delivery chemistry, intracellular drug delivery capabilities, and a search and evaluation group within ADD.
+Previously, Annette worked for Amgen and Merck in the US, focusing on small molecule and peptide formulations, outsourcing partnerships in China, and in-licensing and partnership evaluations. She contributed to bringing small molecule therapies to market.
+Annette has published over 50 articles, given more than 50 invited presentations, and serves on the editorial boards of the Journal of Pharmaceutical Sciences and Molecular Pharmaceutics. She holds several patents for pharmaceutical technologies.
+A key volunteer in the American Association of Pharmaceutical Scientists (AAPS), Annette was the 2022 president, leading the implementation of the 2021-2025 strategic plan. She was the 2020 co-recipient of the AAPS Alice E. Till Women in Pharmaceutical Science Recognition.
+We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
+Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
+This website uses the following types of services. Learn more from our
+                    Cookie Policy.
+By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+        </is>
+      </c>
       <c r="K25" t="inlineStr">
         <is>
           <t>https://lnp-formulation-process-development-pharma.com/speaker/annette-bak/</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr"/>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>https://lnp-formulation-process-development-pharma.com/wp-content/uploads/sites/241/2025/11/Annette-Bak-300x300.png</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>images/annette_bak.jpg</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-282EB2</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1820,28 +2375,47 @@
           <t>Beam Therapeutics</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Vice President - Delivery Platform Beam Therapeutics
+We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
+Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
+This website uses the following types of services. Learn more from our
+                    Cookie Policy.
+By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+        </is>
+      </c>
       <c r="K26" t="inlineStr">
         <is>
           <t>https://lnp-formulation-process-development-pharma.com/speaker/luis-brito/</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr"/>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>https://lnp-formulation-process-development-pharma.com/wp-content/uploads/sites/241/2025/11/Luis-Brito-300x300.png</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>images/luis_brito.jpg</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-3FC9E8</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>LNP Formulation</t>
+          <t>Gene Therapy Conference</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Pharma Formulation</t>
+          <t>Gene Therapy</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1856,36 +2430,54 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Ching</t>
+          <t>Damir</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Ching Kim Tye</t>
+          <t>Damir Simic</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Head of DP Platform and Early Clinical Development</t>
+          <t>Executive Director</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Sanofi</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr"/>
+          <t>Astellas Pharma</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
+Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
+This website uses the following types of services. Learn more from our
+                    Cookie Policy.
+By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+        </is>
+      </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>https://lnp-formulation-process-development-pharma.com/speaker/ching-kim-tye/</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr"/>
+          <t>https://genetherapy-conference.com/speaker/damir-simic/</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>https://genetherapy-conference.com/wp-content/uploads/sites/227/2025/11/Damir-Simic-1-300x300.png</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>images/damir_simic.jpg</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-3FC9E8</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1910,36 +2502,38 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Damir</t>
+          <t>Jorge</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Damir Simic</t>
+          <t>Jorge Santiago-Ortiz</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Executive Director</t>
+          <t>Senior Director - Chemistry, Manufacturing &amp; Controls</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Astellas Pharma</t>
+          <t>Apertura Gene Therapy</t>
         </is>
       </c>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
-          <t>https://genetherapy-conference.com/speaker/damir-simic/</t>
+          <t>https://genetherapy-conference.com/speaker/jorge-santiago-ortiz/</t>
         </is>
       </c>
       <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-3FC9E8</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1964,36 +2558,56 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Jorge</t>
+          <t>Devyn</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Jorge Santiago-Ortiz</t>
+          <t>Devyn Smith</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Senior Director - Chemistry, Manufacturing &amp; Controls</t>
+          <t>Chief Executive Officer</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Apertura Gene Therapy</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr"/>
+          <t>Arbor Biotechnologies, Inc.</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Chief Executive Officer Arbor Biotechnologies, Inc.
+Dr. Devyn Smith brings significant cell and gene therapy development and platform expertise from his 20+ year career. Devyn joined Arbor Biotechnologies as Chief Executive Officer on April 27, 2021 after concluding his role as Chief Operating Officer of Sigilon Therapeutics. Prior to Sigilon, Dr. Smith worked in a variety of roles at Pfizer Inc., including COO of the UK-based Neusentis Unit focused on discovering and developing cell therapies. He received his Ph.D. in Genetics from Harvard Medical School. He is an inventor on multiple patents and has published in leading scientific journals throughout his career. Dr. Smith is a board member and officer for ARM (Alliance for Regenerative Medicine), the cell and gene therapy industry group
+We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
+Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
+This website uses the following types of services. Learn more from our
+                    Cookie Policy.
+By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+        </is>
+      </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>https://genetherapy-conference.com/speaker/jorge-santiago-ortiz/</t>
-        </is>
-      </c>
-      <c r="L29" t="inlineStr"/>
+          <t>https://genetherapy-conference.com/speaker/devyn-smith/</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>https://genetherapy-conference.com/wp-content/uploads/sites/227/2025/11/62945-Speaker-Photos-10-300x300.png</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>images/devyn_smith.jpg</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-3FC9E8</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2018,36 +2632,56 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Devyn</t>
+          <t>Hebe</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Devyn Smith</t>
+          <t>Hebe Sun</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Chief Executive Officer</t>
+          <t>Associate Director, CDx/IVD Regulatory Affairs</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Arbor Biotechnologies, Inc.</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr"/>
+          <t>Regeneron Pharmaceuticals</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Associate Director, CDx/IVD Regulatory Affairs Regeneron Pharmaceuticals
+Hebe Sun, Regulatory Affairs Associate Director in Regeneron, contributed to the CDx/IVD co-development in multiple gene therapy programs in Regeneron. Before Regeneron, she has multiple years of regulatory experience in medical device and IVD industry.
+We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
+Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
+This website uses the following types of services. Learn more from our
+                    Cookie Policy.
+By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+        </is>
+      </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>https://genetherapy-conference.com/speaker/devyn-smith/</t>
-        </is>
-      </c>
-      <c r="L30" t="inlineStr"/>
+          <t>https://genetherapy-conference.com/speaker/hebe-sun/</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>https://genetherapy-conference.com/wp-content/uploads/sites/227/2025/11/62945-Speaker-Photos-11-300x300.png</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>images/hebe_sun.jpg</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-3FC9E8</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2072,36 +2706,56 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Hebe</t>
+          <t>Tassos</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Hebe Sun</t>
+          <t>Tassos Georgiadis</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Associate Director, CDx/IVD Regulatory Affairs</t>
+          <t>Senior VP, Discovery &amp; Preclinical Development</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Regeneron Pharmaceuticals</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr"/>
+          <t>MeiraGTx</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Senior VP, Discovery &amp; Preclinical Development MeiraGTx
+Tassos has been working on retinal gene therapy for 25 years. He has developed AAV vectors for a range of indications that are currently in clinical development (Ph1/2, Ph3, pre-commercialization). He is currently Senior Vice President, Discovery &amp; Preclinical Development at MeiraGTx establishing a multi-platform assessment strategy for drug product candidate screening, with a focus on retina and CNS.
+We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
+Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
+This website uses the following types of services. Learn more from our
+                    Cookie Policy.
+By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+        </is>
+      </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>https://genetherapy-conference.com/speaker/hebe-sun/</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr"/>
+          <t>https://genetherapy-conference.com/speaker/tassos-georgiadis/</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>https://genetherapy-conference.com/wp-content/uploads/sites/227/2025/11/62945-Speaker-Photos-27-300x300.png</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>images/tassos_georgiadis.jpg</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-3FC9E8</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2126,36 +2780,56 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Tassos</t>
+          <t>Casey</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Tassos Georgiadis</t>
+          <t>Casey Maguire</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Senior VP, Discovery &amp; Preclinical Development</t>
+          <t>Investigator &amp; Associate Professor</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>MeiraGTx</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr"/>
+          <t>Harvard Medical School</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Investigator &amp; Associate Professor Harvard Medical School
+Casey A. Maguire obtained a B.S. in Microbiology from the University of Maine in 2000 and a PhD from the Department of Microbiology and Immunology at the University of Rochester School of Medicine and Dentistry in 2006. He was a postdoctoral fellow at the MGH from 2006-2010. He was next an Instructor from 2010-2013 and Assistant Professor from 2013-2019. Currently he is an Associate Professor of Neurology at Harvard Medical School with his laboratory located at the MGH Research Institute.
+We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
+Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
+This website uses the following types of services. Learn more from our
+                    Cookie Policy.
+By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+        </is>
+      </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>https://genetherapy-conference.com/speaker/tassos-georgiadis/</t>
-        </is>
-      </c>
-      <c r="L32" t="inlineStr"/>
+          <t>https://genetherapy-conference.com/speaker/casey-maguire/</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>https://genetherapy-conference.com/wp-content/uploads/sites/227/2025/11/62945-Speaker-Photos-4-300x300.png</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>images/casey_maguire.jpg</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-3FC9E8</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2180,36 +2854,55 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Casey</t>
+          <t>Lindsay</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Casey Maguire</t>
+          <t>Lindsay Marjoram</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Investigator &amp; Associate Professor</t>
+          <t>CSO</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Harvard Medical School</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr"/>
+          <t>Barth Syndrome Foundation Inc</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Lindsay Marjoram, PhD is the Director of Research for the Barth Syndrome Foundation, which is dedicated to advocacy and advancing research for the development of treatments and, one day, cures for this ultra-rare disease. Dr. Marjoram has a background in developmental biology and a vested interest in rare disease research. Prior to joining the Barth Syndrome Foundation, Dr. Marjoram worked for a pre-clinical contract research organization specialized in ophthalmology where she gained extensive experience in cutting edge gene therapies and rare diseases impacting vision loss
+We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
+Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
+This website uses the following types of services. Learn more from our
+                    Cookie Policy.
+By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+        </is>
+      </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>https://genetherapy-conference.com/speaker/casey-maguire/</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr"/>
+          <t>https://genetherapy-conference.com/speaker/lindsay-marjoram/</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>https://genetherapy-conference.com/wp-content/uploads/sites/227/2025/11/62945-Speaker-Photos-16-300x300.png</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>images/lindsay_marjoram.jpg</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>CONF-3FC9E8</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2234,85 +2927,50 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Lindsay</t>
+          <t>Susan</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Lindsay Marjoram</t>
+          <t>Susan serrano</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>CSO</t>
+          <t>Senior Director, Market Access Strategy and Value Communication</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Barth Syndrome Foundation Inc</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr"/>
+          <t>Intellia Therapeutics</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Senior Director, Market Access Strategy and Value Communication Intellia Therapeutics
+We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
+Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
+This website uses the following types of services. Learn more from our
+                    Cookie Policy.
+By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+        </is>
+      </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>https://genetherapy-conference.com/speaker/lindsay-marjoram/</t>
-        </is>
-      </c>
-      <c r="L34" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Gene Therapy Conference</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Gene Therapy</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>Susan</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>Susan serrano</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>Senior Director, Market Access Strategy and Value Communication</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>Intellia Therapeutics</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr">
-        <is>
           <t>https://genetherapy-conference.com/speaker/susan-serrano/</t>
         </is>
       </c>
-      <c r="L35" t="inlineStr"/>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>https://genetherapy-conference.com/wp-content/uploads/sites/227/2025/11/Susan-Serrano-300x300.png</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>images/susan_serrano.jpg</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
added strict garbage filter for speaker bios
</commit_message>
<xml_diff>
--- a/conference_data.xlsx
+++ b/conference_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N34"/>
+  <dimension ref="A1:N26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -536,14 +536,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Thank you to our speakers, sponsors, and delegates who joined us in Boston for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
-Tomi is an entrepreneurial drug hunter with &gt;40 years of industrial experience in both large pharma and biotech. He has three marketed drugs and &gt;670 scientific publications, patents, and presentations (primarily focused on peptide drug discovery). Tomi is the Founding President of the Peptide Drug Hunting Consortium.
-This your chance to hear from pioneering executive leaders the peptide space who will discuss their ambitions, strategies and challenges for peptide discovery, targets. indications and development of next generation of peptide drugs.
-We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
-Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
-This website uses the following types of services. Learn more from our
-                    Cookie Policy.
-By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+          <t>Tomi is an entrepreneurial drug hunter with &gt;40 years of industrial experience in both large pharma and biotech. He has three marketed drugs and &gt;670 scientific publications, patents, and presentations (primarily focused on peptide drug discovery). Tomi is the Founding President of the Peptide Drug Hunting Consortium.</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -611,13 +604,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Thank you to our speakers, sponsors, and delegates who joined us in Boston for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
-Philip Jonas Sassene has a strong track record in drug delivery. He has 15+ years of experience in enabling formulations with particular emphasis on enabling formulation strategies for oral delivery of peptides &amp; proteins. He is currently employed as a Scientific Director within oral delivery technologies at Novo Nordisk A/S.
-We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
-Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
-This website uses the following types of services. Learn more from our
-                    Cookie Policy.
-By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+          <t>Philip Jonas Sassene has a strong track record in drug delivery. He has 15+ years of experience in enabling formulations with particular emphasis on enabling formulation strategies for oral delivery of peptides &amp; proteins. He is currently employed as a Scientific Director within oral delivery technologies at Novo Nordisk A/S.</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -685,13 +672,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Thank you to our speakers, sponsors, and delegates who joined us in Boston for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
-The biopharmaceutical sector continues to innovate peptide discovery innovations, from new macrocycles to new delivery methods and are thriving on strategic alliances, which allow for cross-functional sharing of knowledge, and experience to advance peptide drugs to patients faster. Hear first-hand how investors and key biotechs are keeping up with the peptide momentum through investments, alliances and collaborations.
-We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
-Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
-This website uses the following types of services. Learn more from our
-                    Cookie Policy.
-By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+          <t>The biopharmaceutical sector continues to innovate peptide discovery innovations, from new macrocycles to new delivery methods and are thriving on strategic alliances, which allow for cross-functional sharing of knowledge, and experience to advance peptide drugs to patients faster. Hear first-hand how investors and key biotechs are keeping up with the peptide momentum through investments, alliances and collaborations.</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -759,13 +740,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Thank you to our speakers, sponsors, and delegates who joined us in Boston for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
-Bradley L. Pentelute is a Professor of Chemistry at MIT (https://pentelutelabmit.com). He is also an Associate Member, Broad Institute of Harvard and MIT, an Extramural Member of the MIT Koch Cancer Institute, and Member, Center for Environmental Health Sciences MIT. He received his undergraduate degree in Psychology and Chemistry from the University of Southern California, and his M.S and Ph.D. in Organic Chemistry from the University of Chicago with Prof. Steve Kent. He was a postdoctoral fellow in the laboratory of Dr. R. John Collier at Harvard Medical School, Microbiology.
-We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
-Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
-This website uses the following types of services. Learn more from our
-                    Cookie Policy.
-By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+          <t>Bradley L. Pentelute is a Professor of Chemistry at MIT (https://pentelutelabmit.com). He is also an Associate Member, Broad Institute of Harvard and MIT, an Extramural Member of the MIT Koch Cancer Institute, and Member, Center for Environmental Health Sciences MIT. He received his undergraduate degree in Psychology and Chemistry from the University of Southern California, and his M.S and Ph.D. in Organic Chemistry from the University of Chicago with Prof. Steve Kent. He was a postdoctoral fellow in the laboratory of Dr. R. John Collier at Harvard Medical School, Microbiology.</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -833,17 +808,11 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Thank you to our speakers, sponsors, and delegates who joined us in Boston for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
-Annette Bak, Ph.D., MBA, leads Advanced Drug Delivery (ADD) at AstraZeneca and serves on the Pharmaceutical Sciences leadership team. ADD, a global organization with over 100 employees in Sweden, UK, and US, aims to transform diverse modalities into investigational medicines.
+          <t>Annette Bak, Ph.D., MBA, leads Advanced Drug Delivery (ADD) at AstraZeneca and serves on the Pharmaceutical Sciences leadership team. ADD, a global organization with over 100 employees in Sweden, UK, and US, aims to transform diverse modalities into investigational medicines.
 Since joining AstraZeneca in 2016, Annette has delivered various synthetic modalities and mRNA drug delivery systems for preclinical and clinical studies. She has also built delivery chemistry, intracellular drug delivery capabilities, and a search and evaluation group within ADD.
 Previously, Annette worked for Amgen and Merck in the US, focusing on small molecule and peptide formulations, outsourcing partnerships in China, and in-licensing and partnership evaluations. She contributed to bringing small molecule therapies to market.
 Annette has published over 50 articles, given more than 50 invited presentations, and serves on the editorial boards of the Journal of Pharmaceutical Sciences and Molecular Pharmaceutics. She holds several patents for pharmaceutical technologies.
-A key volunteer in the American Association of Pharmaceutical Scientists (AAPS), Annette was the 2022 president, leading the implementation of the 2021-2025 strategic plan. She was the 2020 co-recipient of the AAPS Alice E. Till Women in Pharmaceutical Science Recognition.
-We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
-Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
-This website uses the following types of services. Learn more from our
-                    Cookie Policy.
-By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+A key volunteer in the American Association of Pharmaceutical Scientists (AAPS), Annette was the 2022 president, leading the implementation of the 2021-2025 strategic plan. She was the 2020 co-recipient of the AAPS Alice E. Till Women in Pharmaceutical Science Recognition.</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -911,14 +880,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Thank you to our speakers, sponsors, and delegates who joined us in Boston for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
-Thomas von Erlach, PhD co-founded Vivtex and joined as its Chief Scientific Officer when Vivtex was formed as a MIT spin-off in 2018. Prior to that he led the interdisciplinary efforts around gastrointestinal model systems for oral drug delivery applications at the Laboratory of Prof. Robert Langer and Prof. Giovanni Traverso at MIT. Dr von Erlach obtained his PhD from Imperial College London in Bioengineering and a BSc and MSc in Biochemistry and Biotechnology from ETH Zurich in Switzerland. His research interest include advanced in vitro models for drug development, oral drug delivery and gastrointestinal pharmacology. His work is published in several high impact journals such as Nature Materials, Nature Biomedical Engineering, and Nature Communications.
-The biopharmaceutical sector continues to innovate peptide discovery innovations, from new macrocycles to new delivery methods and are thriving on strategic alliances, which allow for cross-functional sharing of knowledge, and experience to advance peptide drugs to patients faster. Hear first-hand how investors and key biotechs are keeping up with the peptide momentum through investments, alliances and collaborations.
-We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
-Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
-This website uses the following types of services. Learn more from our
-                    Cookie Policy.
-By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+          <t>Thomas von Erlach, PhD co-founded Vivtex and joined as its Chief Scientific Officer when Vivtex was formed as a MIT spin-off in 2018. Prior to that he led the interdisciplinary efforts around gastrointestinal model systems for oral drug delivery applications at the Laboratory of Prof. Robert Langer and Prof. Giovanni Traverso at MIT. Dr von Erlach obtained his PhD from Imperial College London in Bioengineering and a BSc and MSc in Biochemistry and Biotechnology from ETH Zurich in Switzerland. His research interest include advanced in vitro models for drug development, oral drug delivery and gastrointestinal pharmacology. His work is published in several high impact journals such as Nature Materials, Nature Biomedical Engineering, and Nature Communications.</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -986,15 +948,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Thank you to our speakers, sponsors, and delegates who joined us in Boston for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
-Shelley Allen is an accomplished drug discovery leader with more than 25 years of experience in medicinal chemistry. She has a proven history of building and leading successful teams in both biotech and pharma, consistently delivering high-quality drug candidates with a strong sense of urgency. Shelley served as the Head of Drug Discovery at Nimble Therapeutics until its acquisition by AbbVie earlier this year. She now continues her impactful work at AbbVie, contributing to the discovery and development of peptide programs within the Immuno-Pharmacology &amp; Peptide Discovery group.
-Practical Approaches to Characterize ADME &amp; Design Translatable In Vitro &amp; In Vivo PK/PD Studies with Jianzhong Wen
-Improving Permeating Agent Performance to Achieve Successful Peptide Oral Bioavailability with Shelley Allen
-We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
-Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
-This website uses the following types of services. Learn more from our
-                    Cookie Policy.
-By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+          <t>Shelley Allen is an accomplished drug discovery leader with more than 25 years of experience in medicinal chemistry. She has a proven history of building and leading successful teams in both biotech and pharma, consistently delivering high-quality drug candidates with a strong sense of urgency. Shelley served as the Head of Drug Discovery at Nimble Therapeutics until its acquisition by AbbVie earlier this year. She now continues her impactful work at AbbVie, contributing to the discovery and development of peptide programs within the Immuno-Pharmacology &amp; Peptide Discovery group.</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1062,13 +1016,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Thank you to our speakers, sponsors, and delegates who joined us in Boston for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
-Qook Lee joined the BioTDR group at Eli Lilly as a Research Scientist in 2017 and currently serves as a Research Advisor (Engineer) in Lilly Genetic Medicine at the Lilly Seaport Innovation Center. His work has focused on developing oral GG and GGG delivery platforms using hydrogels, polymeric particles, minitablets, and other technologies for extended drug delivery platform. He has also contributed to the evaluation of formulation and analytical method development in the mRNA-LNP-based protein replacement therapeutic area, gene editing and LNP production process development and supported large animal study productions.
-We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
-Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
-This website uses the following types of services. Learn more from our
-                    Cookie Policy.
-By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+          <t>Qook Lee joined the BioTDR group at Eli Lilly as a Research Scientist in 2017 and currently serves as a Research Advisor (Engineer) in Lilly Genetic Medicine at the Lilly Seaport Innovation Center. His work has focused on developing oral GG and GGG delivery platforms using hydrogels, polymeric particles, minitablets, and other technologies for extended drug delivery platform. He has also contributed to the evaluation of formulation and analytical method development in the mRNA-LNP-based protein replacement therapeutic area, gene editing and LNP production process development and supported large animal study productions.</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1134,31 +1082,14 @@
           <t>Johnson &amp; Johnson</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>Thank you to our speakers, sponsors, and delegates who joined us in Boston for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
-We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
-Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
-This website uses the following types of services. Learn more from our
-                    Cookie Policy.
-By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
-        </is>
-      </c>
+      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
           <t>https://peptide-based-therapeutics-summit.com/speaker/sumit-arora/</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>https://peptide-based-therapeutics-summit.com/wp-content/uploads/sites/255/2025/11/Sumit-Arora-300x300.png</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>images/sumit_arora.jpg</t>
-        </is>
-      </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
@@ -1209,13 +1140,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Thank you to our speakers, sponsors, and delegates who joined us in Boston for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
-Dr. Maria Fawaz is an Associate Principal Scientist in Pharmacokinetics, Dynamics, Metabolism &amp; Bioanalytics at Merck Research Laboratories, West Point, PA. As a DMPK principal investigator, Maria supports various peptide modalities, guiding design strategies in the early discovery space, lead optimization, and also supports clinical-stage programs. Maria has extensive experience in cyclic peptide metabolite identification, where she co-discovered novel analytical strategies of unambiguously identifying regions in the cyclic peptide sequence susceptible to amide hydrolysis by proteases. At Merck, Maria is also working with external collaborators and various funding organizations. Maria holds a PhD degree in Medicinal Chemistry from the University of Michigan. Her doctoral research was focused on the design and synthesis of high-density lipoproteins (sHDL) composed of ApoA-I mimetic peptides and phospholipids for the treatment of Niemann-Pick diseases and atherosclerosis. Maria is passionate about mentoring junior scientists and she is actively engaged in student and postdoc career outreach at various universities.
-We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
-Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
-This website uses the following types of services. Learn more from our
-                    Cookie Policy.
-By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+          <t>Dr. Maria Fawaz is an Associate Principal Scientist in Pharmacokinetics, Dynamics, Metabolism &amp; Bioanalytics at Merck Research Laboratories, West Point, PA. As a DMPK principal investigator, Maria supports various peptide modalities, guiding design strategies in the early discovery space, lead optimization, and also supports clinical-stage programs. Maria has extensive experience in cyclic peptide metabolite identification, where she co-discovered novel analytical strategies of unambiguously identifying regions in the cyclic peptide sequence susceptible to amide hydrolysis by proteases. At Merck, Maria is also working with external collaborators and various funding organizations. Maria holds a PhD degree in Medicinal Chemistry from the University of Michigan. Her doctoral research was focused on the design and synthesis of high-density lipoproteins (sHDL) composed of ApoA-I mimetic peptides and phospholipids for the treatment of Niemann-Pick diseases and atherosclerosis. Maria is passionate about mentoring junior scientists and she is actively engaged in student and postdoc career outreach at various universities.</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1283,19 +1208,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Why Not Join Us for the Next Event in the World Biomarkers &amp; Diagnostics Series?
-Discover the 16th World Clinical Biomarkers &amp; CDx Summit here
-Thank you to our speakers, sponsors, and delegates who joined us in London for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
-Why Not Join Us for the Next Event in the World Biomarkers &amp; Diagnostics Series?
-Discover the 16th World Clinical Biomarkers &amp; CDx Summit here
-Thank you to our speakers, sponsors, and delegates who joined us in London for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
-Director - Medical, Translational &amp; Computational Pathology GSK
-Monika Lamba Saini is a highly skilled professional currently serving as the Global Translational Pathology Leader at ADC Therapeutics since August 2024, where strategic leadership is provided to enhance the understanding of diseases and to implement translational research strategies for developing novel therapeutics. In addition, Monika is an Education Committee Member at the Digital Pathology Association, contributing to webinars and academic content. Prior experience includes roles as Director of Digital Pathology Innovation and Pathology Research Scientist at IQVIA Laboratories, focusing on digital pathology and AI-driven trials, and as a Pathologist and Principal Investigator at CellCarta, specializing in histopathological evaluations of cancers and immune-oncology therapies. Monika also has an extensive academic background, including a PhD in Biomedical Sciences and a Doctor of Medicine degree in Pathology from esteemed institutions.
-We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
-Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
-This website uses the following types of services. Learn more from our
-                    Cookie Policy.
-By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+          <t>Monika Lamba Saini is a highly skilled professional currently serving as the Global Translational Pathology Leader at ADC Therapeutics since August 2024, where strategic leadership is provided to enhance the understanding of diseases and to implement translational research strategies for developing novel therapeutics. In addition, Monika is an Education Committee Member at the Digital Pathology Association, contributing to webinars and academic content. Prior experience includes roles as Director of Digital Pathology Innovation and Pathology Research Scientist at IQVIA Laboratories, focusing on digital pathology and AI-driven trials, and as a Pathologist and Principal Investigator at CellCarta, specializing in histopathological evaluations of cancers and immune-oncology therapies. Monika also has an extensive academic background, including a PhD in Biomedical Sciences and a Doctor of Medicine degree in Pathology from esteemed institutions.</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1363,19 +1276,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Why Not Join Us for the Next Event in the World Biomarkers &amp; Diagnostics Series?
-Discover the 16th World Clinical Biomarkers &amp; CDx Summit here
-Thank you to our speakers, sponsors, and delegates who joined us in London for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
-Why Not Join Us for the Next Event in the World Biomarkers &amp; Diagnostics Series?
-Discover the 16th World Clinical Biomarkers &amp; CDx Summit here
-Thank you to our speakers, sponsors, and delegates who joined us in London for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
-Head of Global Commercial Biomarkers &amp; Diagnostics Amgen
-EK Kim is the Global Head of Commercial Biomarkers and Diagnostics at Amgen, where she leads the commercialization and launch strategy for diagnostic and patient identification tools across oncology, cardiovascular, inflammation, and rare disease. She has held leadership roles across commercial and development functions and has directed global readiness for multiple integrated medicine and diagnostic launches. Prior to Amgen, EK held senior roles at AstraZeneca, Personal Genome Diagnostics (PGDx), Roche Diagnostics, and Ventana Medical Systems, where she advanced precision medicine strategies that supported global brand planning, development and regulatory planning, and commercialization.
-We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
-Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
-This website uses the following types of services. Learn more from our
-                    Cookie Policy.
-By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+          <t>EK Kim is the Global Head of Commercial Biomarkers and Diagnostics at Amgen, where she leads the commercialization and launch strategy for diagnostic and patient identification tools across oncology, cardiovascular, inflammation, and rare disease. She has held leadership roles across commercial and development functions and has directed global readiness for multiple integrated medicine and diagnostic launches. Prior to Amgen, EK held senior roles at AstraZeneca, Personal Genome Diagnostics (PGDx), Roche Diagnostics, and Ventana Medical Systems, where she advanced precision medicine strategies that supported global brand planning, development and regulatory planning, and commercialization.</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1443,24 +1344,13 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Why Not Join Us for the Next Event in the World Biomarkers &amp; Diagnostics Series?
-Discover the 16th World Clinical Biomarkers &amp; CDx Summit here
-Thank you to our speakers, sponsors, and delegates who joined us in London for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
-Why Not Join Us for the Next Event in the World Biomarkers &amp; Diagnostics Series?
-Discover the 16th World Clinical Biomarkers &amp; CDx Summit here
-Thank you to our speakers, sponsors, and delegates who joined us in London for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
-Angela is an Inspirational leader with a demonstrated history of working previously in the NHS for over 42 years, as DCSO and in Genetics and Genomics, as the Scientific Director of a Regional Genomics Service and Clinical Programme Director of the NW Coast Genomic Medicine Centre.
+          <t>Angela is an Inspirational leader with a demonstrated history of working previously in the NHS for over 42 years, as DCSO and in Genetics and Genomics, as the Scientific Director of a Regional Genomics Service and Clinical Programme Director of the NW Coast Genomic Medicine Centre.
 She retired from the post of the Deputy Chief Scientific Officer (DCSO) for NHS England in October 2023, after holding the position for 5 yrs. Angela is now the President of BIVDA having taken up this role in December 2023. She is an influential, collaborative team leader with a proven record in Clinical Research, Medical Education, Mentoring and Coaching, in Life Sciences.
 Angela has a strong financial acumen and is a strategic leadership expert. She is passionate about quality assurance, safety and regulation in Science and in particular Genetics and Genomics, her area of expertise. She graduated from University College London and is a Fellow of the Royal College of Pathologists and an honorary Fellow of the Academy for Healthcare Science.
 She had the pleasure of being the President of the BSGM, Chairman of the RCPath Genetics and Reproductive Medicines Specialist Advisory Committee and was RCPath’s Scientific Lead before taking on the role of DCSO.
 In 2014, Angela was named as one of HSJ’s top 50 Inspirational Women. In 2015, she was awarded NHS Healthcare Scientist of the Year, and in 2016, was honoured in Her Majesty the Queen’s 90th Birthday Honours List as a Member of the Order of the British Empire for Research and Mentoring Students.
 In 2019, she was included in the Pathologist Power list as one of the top 100 trailblazers. In 2021, Angela was delighted to be approved as an Honorary Fellow of IPEM. In 2022 her leadership journey was published in Snapshots of Women in COG. In 2023, the AHCS again recognised her contribution to education and training with a second Fellowship.
-In 2023, Angela was nominated as a Woman of the Year by the Women Leaders Network. Angela is an inclusive, compassionate and kind leader with a broad experience of working across the healthcare system, and in all her endeavours strives to bring out the best in all those she works with.
-We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
-Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
-This website uses the following types of services. Learn more from our
-                    Cookie Policy.
-By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+In 2023, Angela was nominated as a Woman of the Year by the Women Leaders Network. Angela is an inclusive, compassionate and kind leader with a broad experience of working across the healthcare system, and in all her endeavours strives to bring out the best in all those she works with.</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1528,19 +1418,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Why Not Join Us for the Next Event in the World Biomarkers &amp; Diagnostics Series?
-Discover the 16th World Clinical Biomarkers &amp; CDx Summit here
-Thank you to our speakers, sponsors, and delegates who joined us in London for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
-Why Not Join Us for the Next Event in the World Biomarkers &amp; Diagnostics Series?
-Discover the 16th World Clinical Biomarkers &amp; CDx Summit here
-Thank you to our speakers, sponsors, and delegates who joined us in London for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
-Senior Director, Global Regulatory Affairs Diagnostics Eli Lilly &amp; Co.
-Nicole Chaves Petronzi is Senior Director of Global Regulatory Affairs Diagnostics at Lilly. With extensive experience in in-vitro diagnostics and pharmaceutical regulatory strategy, Nicole has led global initiatives to implement the EU IVDR and harmonize compliance across multiple markets. Her work focuses on integrating diagnostics into pharmaceutical development, driving collaboration between Regulatory Affairs, Quality, Clinical, and Laboratory teams to accelerate innovation and patient access. Nicole is recognized for her ability to navigate complex regulatory landscapes and transform compliance into a strategic advantage for diagnostics in pharma.
-We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
-Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
-This website uses the following types of services. Learn more from our
-                    Cookie Policy.
-By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+          <t>Nicole Chaves Petronzi is Senior Director of Global Regulatory Affairs Diagnostics at Lilly. With extensive experience in in-vitro diagnostics and pharmaceutical regulatory strategy, Nicole has led global initiatives to implement the EU IVDR and harmonize compliance across multiple markets. Her work focuses on integrating diagnostics into pharmaceutical development, driving collaboration between Regulatory Affairs, Quality, Clinical, and Laboratory teams to accelerate innovation and patient access. Nicole is recognized for her ability to navigate complex regulatory landscapes and transform compliance into a strategic advantage for diagnostics in pharma.</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1608,20 +1486,9 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Why Not Join Us for the Next Event in the World Biomarkers &amp; Diagnostics Series?
-Discover the 16th World Clinical Biomarkers &amp; CDx Summit here
-Thank you to our speakers, sponsors, and delegates who joined us in London for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
-Why Not Join Us for the Next Event in the World Biomarkers &amp; Diagnostics Series?
-Discover the 16th World Clinical Biomarkers &amp; CDx Summit here
-Thank you to our speakers, sponsors, and delegates who joined us in London for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
-Dr Catherine Mela is Head of Biomarker Operations, within GSK. In her role, Catherine is accountable for leading the Scientific Operations and Data Operations teams, driving the execution of precision medicine project strategies with efficiency and quality.
+          <t>Dr Catherine Mela is Head of Biomarker Operations, within GSK. In her role, Catherine is accountable for leading the Scientific Operations and Data Operations teams, driving the execution of precision medicine project strategies with efficiency and quality.
 Catherine has gained broad experience in laboratory and bio-sample operations, while leading Human Biological Sample operational and governance teams in AstraZeneca and Roche.
-Prior to working in pharma, Catherine’s background was in Clinical research within the NHS. She holds a PhD from Imperial College on ‘The impact of treatment strategies on immune responses in HIV-1 infection’. Catherine is a fellow of the institute of leadership and is passionate about professional development, mentorship and creating a supportive environment for individuals within her teams.
-We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
-Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
-This website uses the following types of services. Learn more from our
-                    Cookie Policy.
-By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+Prior to working in pharma, Catherine’s background was in Clinical research within the NHS. She holds a PhD from Imperial College on ‘The impact of treatment strategies on immune responses in HIV-1 infection’. Catherine is a fellow of the institute of leadership and is passionate about professional development, mentorship and creating a supportive environment for individuals within her teams.</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1689,20 +1556,8 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Why Not Join Us for the Next Event in the World Biomarkers &amp; Diagnostics Series?
-Discover the 16th World Clinical Biomarkers &amp; CDx Summit here
-Thank you to our speakers, sponsors, and delegates who joined us in London for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
-Why Not Join Us for the Next Event in the World Biomarkers &amp; Diagnostics Series?
-Discover the 16th World Clinical Biomarkers &amp; CDx Summit here
-Thank you to our speakers, sponsors, and delegates who joined us in London for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
-Scientific-Regulatory Assessor Targeted &amp; Personalized Biomedicines Paul-Ehrlich-Institut, National Competent Authority for Medicinal Products &amp; CDx Devices
-Jörg Engelbergs is currently working for the Paul-Ehrlich-Institut (PEI), German National Competent Authority for Medicinal Products and CDx devices, as a scientific-regulatory assessor (Quality, Non-Clinic, Biomarkers, CDx). He is involved in the European process of marketing authorization and life cycle of predictive biomarker guided biopharmaceuticals comprising scientific assessments and advices. Further tasks are assessments of CTR conformity of clinical trials and IVDR conformity of associated CDx performance studies. He is also responsible for the technical, procedural and scientific implementation of the new responsibility of PEI for CDx performance studies. At the European level he is member of several CDx related European working groups, e.g. EMA CHMP/CAT CDx Expert Group (Co-Chair), EMA Methodology Working Party, EMA SIA PGx (Leadership Team), and EU COMBINE Project.
-He holds a Diploma in biology and a PhD. He has extensive experience as scientific project leader in cancer research at the West German Cancer Center (WTZE) and in neuropharmacology research, including R&amp;D of diagnostic/predictive biomarkers and assays, as well as in the establishment and management of a central clinical genotyping service center at the Medical Faculty of the University of Essen, Germany.
-We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
-Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
-This website uses the following types of services. Learn more from our
-                    Cookie Policy.
-By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+          <t>Jörg Engelbergs is currently working for the Paul-Ehrlich-Institut (PEI), German National Competent Authority for Medicinal Products and CDx devices, as a scientific-regulatory assessor (Quality, Non-Clinic, Biomarkers, CDx). He is involved in the European process of marketing authorization and life cycle of predictive biomarker guided biopharmaceuticals comprising scientific assessments and advices. Further tasks are assessments of CTR conformity of clinical trials and IVDR conformity of associated CDx performance studies. He is also responsible for the technical, procedural and scientific implementation of the new responsibility of PEI for CDx performance studies. At the European level he is member of several CDx related European working groups, e.g. EMA CHMP/CAT CDx Expert Group (Co-Chair), EMA Methodology Working Party, EMA SIA PGx (Leadership Team), and EU COMBINE Project.
+He holds a Diploma in biology and a PhD. He has extensive experience as scientific project leader in cancer research at the West German Cancer Center (WTZE) and in neuropharmacology research, including R&amp;D of diagnostic/predictive biomarkers and assays, as well as in the establishment and management of a central clinical genotyping service center at the Medical Faculty of the University of Essen, Germany.</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1770,19 +1625,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Why Not Join Us for the Next Event in the World Biomarkers &amp; Diagnostics Series?
-Discover the 16th World Clinical Biomarkers &amp; CDx Summit here
-Thank you to our speakers, sponsors, and delegates who joined us in London for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
-Why Not Join Us for the Next Event in the World Biomarkers &amp; Diagnostics Series?
-Discover the 16th World Clinical Biomarkers &amp; CDx Summit here
-Thank you to our speakers, sponsors, and delegates who joined us in London for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
-Honorary Medical Oncologist &amp; Professor of Oncology The Newcastle upon Tyne Hospitals NHS Foundation Trust &amp; Newcastle University
-Professor Greystoke joined Newcastle University and the Northern Centre for Cancer Care in 2014 after 8 years spent at the University of Manchester/ Christie NHS Trust. He is one of 4 consultants that run the Sir Bobby Robson Early Clinical Trials Centre at the Freeman hospital in Newcastle,and has a special interest in the development of new anti-cancer drugs for patients with lung cancer. He leads systemic therapy research for NSCLC in the North-East, with a portfolio of Phase I-IV studies. In addition he is the Clinical Director for Cancer for the Yorkshire, Hull and North East England Genomic Medicine Service and led the NHSE pilot assessing the cost-effectiveness of cfDNA in patients presenting with advanced lung cancer. He is the Joint Chief Investigator of the CONCORDE platform (adding in new drugs to radical radiotherapy in lung cancer), and leads the Pharmacodynamic Biomarker team at Newcastle University Cancer.
-We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
-Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
-This website uses the following types of services. Learn more from our
-                    Cookie Policy.
-By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+          <t>Professor Greystoke joined Newcastle University and the Northern Centre for Cancer Care in 2014 after 8 years spent at the University of Manchester/ Christie NHS Trust. He is one of 4 consultants that run the Sir Bobby Robson Early Clinical Trials Centre at the Freeman hospital in Newcastle,and has a special interest in the development of new anti-cancer drugs for patients with lung cancer. He leads systemic therapy research for NSCLC in the North-East, with a portfolio of Phase I-IV studies. In addition he is the Clinical Director for Cancer for the Yorkshire, Hull and North East England Genomic Medicine Service and led the NHSE pilot assessing the cost-effectiveness of cfDNA in patients presenting with advanced lung cancer. He is the Joint Chief Investigator of the CONCORDE platform (adding in new drugs to radical radiotherapy in lung cancer), and leads the Pharmacodynamic Biomarker team at Newcastle University Cancer.</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1850,19 +1693,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Why Not Join Us for the Next Event in the World Biomarkers &amp; Diagnostics Series?
-Discover the 16th World Clinical Biomarkers &amp; CDx Summit here
-Thank you to our speakers, sponsors, and delegates who joined us in London for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
-Why Not Join Us for the Next Event in the World Biomarkers &amp; Diagnostics Series?
-Discover the 16th World Clinical Biomarkers &amp; CDx Summit here
-Thank you to our speakers, sponsors, and delegates who joined us in London for the summit! If you are interested in the 2027 event, please get in touch at info@hansonwade.com
-Senior Director, Global Precision Medicine Lead Astellas Pharma
-Aino Telaranta-Keerie has worked 20+ years in the pharmaceutical and diagnostic industries, with 10+ years’ experience as Precision Medicine leader in oncology at AstraZeneca and Astellas. She is passionate about optimising CDx partnerships and strategies to ensure successful development of new therapies for patients.
-We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
-Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
-This website uses the following types of services. Learn more from our
-                    Cookie Policy.
-By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+          <t>Aino Telaranta-Keerie has worked 20+ years in the pharmaceutical and diagnostic industries, with 10+ years’ experience as Precision Medicine leader in oncology at AstraZeneca and Astellas. She is passionate about optimising CDx partnerships and strategies to ensure successful development of new therapies for patients.</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1930,14 +1761,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Associate Director - RNA Delivery Sciences GlaxoSmithKline
-Dr. Rushit Lodaya is Associate Director and RNA Delivery Lead at GSK’s RNA Center of Excellence, where he advances delivery platforms for vaccines and infectious diseases. He specializes in Lipid Nanoparticle (LNP) formulation, scale-up process optimization, and the thermostability of multicomponent systems, including mRNA-LNPs. His expertise also extends to vaccine adjuvant formulation and the optimization of novel adjuvants to enhance immune responses. Dr. Lodaya earned his PhD at Northeastern University under the mentorship of Dr. Mansoor Amiji and Dr. Derek O’Hagan, where he developed a strong foundation in nanomedicine and translational vaccine research.
-With immune responses, from anti-PEG and ligand antibodies to component-linked immunogenicity, impacting LNP dosing regimens and limiting clinical success. This workshop will delve into advanced analytics for understanding safety and evaluate innovative solutions to achieve effective repeat dosing.
-We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
-Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
-This website uses the following types of services. Learn more from our
-                    Cookie Policy.
-By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+          <t>Dr. Rushit Lodaya is Associate Director and RNA Delivery Lead at GSK’s RNA Center of Excellence, where he advances delivery platforms for vaccines and infectious diseases. He specializes in Lipid Nanoparticle (LNP) formulation, scale-up process optimization, and the thermostability of multicomponent systems, including mRNA-LNPs. His expertise also extends to vaccine adjuvant formulation and the optimization of novel adjuvants to enhance immune responses. Dr. Lodaya earned his PhD at Northeastern University under the mentorship of Dr. Mansoor Amiji and Dr. Derek O’Hagan, where he developed a strong foundation in nanomedicine and translational vaccine research.</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -2005,14 +1829,8 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Senior Scientist - Drug Product Development Moderna
-Michael “Mike” Smith currently serves as Director of the Emerging Technologies group at Moderna. In his role, Mike leads a cross-disciplinary science and engineering team developing lipid nanoparticle (LNP) formulation platforms for messenger RNA (mRNA). Mike is a self-proclaimed “nanoparticle geek” and has a deep curiosity for the physical chemistry of nanoparticle self-assembly. Leveraging the science of nanoparticle synthesis, the team has built robust scale-up capabilities that service Moderna’s ambitious development portfolio, which includes over 40 drug candidates in active development. Mike and team were major contributors towards the development of Moderna vaccine against SARS-COVID-2 (mRNA-1273). His efforts, together with the Moderna team, were featured in a CNN Hero’s segment and further showcased in NY Magazine (see links below).
-Mike has led numerous scientific and engineering projects over eleven years at Moderna. In years prior, Mike contributed to nanoparticle formulation efforts at Merck that include siRNA LNP and liposomal formulations. Prior to his time in industry, Mike received his PhD from Georgia Tech with a dissertation on the topic of stimuli-responsive hydrogel nanoparticles for therapeutic delivery.
-We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
-Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
-This website uses the following types of services. Learn more from our
-                    Cookie Policy.
-By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+          <t>Michael “Mike” Smith currently serves as Director of the Emerging Technologies group at Moderna. In his role, Mike leads a cross-disciplinary science and engineering team developing lipid nanoparticle (LNP) formulation platforms for messenger RNA (mRNA). Mike is a self-proclaimed “nanoparticle geek” and has a deep curiosity for the physical chemistry of nanoparticle self-assembly. Leveraging the science of nanoparticle synthesis, the team has built robust scale-up capabilities that service Moderna’s ambitious development portfolio, which includes over 40 drug candidates in active development. Mike and team were major contributors towards the development of Moderna vaccine against SARS-COVID-2 (mRNA-1273). His efforts, together with the Moderna team, were featured in a CNN Hero’s segment and further showcased in NY Magazine (see links below).
+Mike has led numerous scientific and engineering projects over eleven years at Moderna. In years prior, Mike contributed to nanoparticle formulation efforts at Merck that include siRNA LNP and liposomal formulations. Prior to his time in industry, Mike received his PhD from Georgia Tech with a dissertation on the topic of stimuli-responsive hydrogel nanoparticles for therapeutic delivery.</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -2080,12 +1898,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Dr. Emma Wang is the chief technology officer and co-founder at YolTech Therapeutics. Her focus is on advancing the non-viral delivery platform to support in vivo gene therapy development through research in novel lipid discovery, product development, process development, characterization as well as GMP manufacture. Prior to joining YolTech, Emma held research positions of growing responsibilities at Providence Therapeutics and Beam Therapeutics. Emma holds a Ph.D. in Chemistry as a member of Prof. Katharina Landfester’s group from Max Planck Institute for Polymer Research in Germany, a M.Eng and B.Eng in Chemical Engineering from McGill University in Canada.
-We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
-Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
-This website uses the following types of services. Learn more from our
-                    Cookie Policy.
-By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+          <t>Dr. Emma Wang is the chief technology officer and co-founder at YolTech Therapeutics. Her focus is on advancing the non-viral delivery platform to support in vivo gene therapy development through research in novel lipid discovery, product development, process development, characterization as well as GMP manufacture. Prior to joining YolTech, Emma held research positions of growing responsibilities at Providence Therapeutics and Beam Therapeutics. Emma holds a Ph.D. in Chemistry as a member of Prof. Katharina Landfester’s group from Max Planck Institute for Polymer Research in Germany, a M.Eng and B.Eng in Chemical Engineering from McGill University in Canada.</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -2151,15 +1964,7 @@
           <t>Tessera Therapeutics</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
-Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
-This website uses the following types of services. Learn more from our
-                    Cookie Policy.
-By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
-        </is>
-      </c>
+      <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
           <t>https://lnp-formulation-process-development-pharma.com/speaker/gulen-tonga/</t>
@@ -2225,14 +2030,8 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Head of DP Platform and Early Clinical Development Sanofi
-Dr. Ching Kim Tye brings two decades of pharmaceutical R&amp;D expertise, specializing in formulation and drug delivery systems. As Head of Drug Product Platform and Early Clinical Development at Sanofi, she leads innovation in mRNA-LNP technology development.
-Currently, Kim spearheads the development of next-generation LNPs with enhanced potency and thermostability for both intramuscular and intranasal delivery routes, advancing candidates into Phase 1 clinical trials. Her comprehensive experience spans from early research through late-stage development, including work with diverse therapeutic modalities—proteins and small molecules at CSL, Pfizer, and Eli Lilly.
-We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
-Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
-This website uses the following types of services. Learn more from our
-                    Cookie Policy.
-By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+          <t>Dr. Ching Kim Tye brings two decades of pharmaceutical R&amp;D expertise, specializing in formulation and drug delivery systems. As Head of Drug Product Platform and Early Clinical Development at Sanofi, she leads innovation in mRNA-LNP technology development.
+Currently, Kim spearheads the development of next-generation LNPs with enhanced potency and thermostability for both intramuscular and intranasal delivery routes, advancing candidates into Phase 1 clinical trials. Her comprehensive experience spans from early research through late-stage development, including work with diverse therapeutic modalities—proteins and small molecules at CSL, Pfizer, and Eli Lilly.</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2304,12 +2103,7 @@
 Since joining AstraZeneca in 2016, Annette has delivered various synthetic modalities and mRNA drug delivery systems for preclinical and clinical studies. She has also built delivery chemistry, intracellular drug delivery capabilities, and a search and evaluation group within ADD.
 Previously, Annette worked for Amgen and Merck in the US, focusing on small molecule and peptide formulations, outsourcing partnerships in China, and in-licensing and partnership evaluations. She contributed to bringing small molecule therapies to market.
 Annette has published over 50 articles, given more than 50 invited presentations, and serves on the editorial boards of the Journal of Pharmaceutical Sciences and Molecular Pharmaceutics. She holds several patents for pharmaceutical technologies.
-A key volunteer in the American Association of Pharmaceutical Scientists (AAPS), Annette was the 2022 president, leading the implementation of the 2021-2025 strategic plan. She was the 2020 co-recipient of the AAPS Alice E. Till Women in Pharmaceutical Science Recognition.
-We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
-Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
-This website uses the following types of services. Learn more from our
-                    Cookie Policy.
-By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+A key volunteer in the American Association of Pharmaceutical Scientists (AAPS), Annette was the 2022 president, leading the implementation of the 2021-2025 strategic plan. She was the 2020 co-recipient of the AAPS Alice E. Till Women in Pharmaceutical Science Recognition.</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2377,12 +2171,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Vice President - Delivery Platform Beam Therapeutics
-We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
-Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
-This website uses the following types of services. Learn more from our
-                    Cookie Policy.
-By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
+          <t>Vice President - Delivery Platform Beam Therapeutics</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2401,576 +2190,6 @@
         </is>
       </c>
       <c r="N26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>CONF-3FC9E8</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Gene Therapy Conference</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Gene Therapy</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Damir</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Damir Simic</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>Executive Director</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>Astellas Pharma</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
-Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
-This website uses the following types of services. Learn more from our
-                    Cookie Policy.
-By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>https://genetherapy-conference.com/speaker/damir-simic/</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>https://genetherapy-conference.com/wp-content/uploads/sites/227/2025/11/Damir-Simic-1-300x300.png</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>images/damir_simic.jpg</t>
-        </is>
-      </c>
-      <c r="N27" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>CONF-3FC9E8</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Gene Therapy Conference</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Gene Therapy</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Jorge</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>Jorge Santiago-Ortiz</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>Senior Director - Chemistry, Manufacturing &amp; Controls</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>Apertura Gene Therapy</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>https://genetherapy-conference.com/speaker/jorge-santiago-ortiz/</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>CONF-3FC9E8</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Gene Therapy Conference</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Gene Therapy</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>Devyn</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>Devyn Smith</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>Chief Executive Officer</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>Arbor Biotechnologies, Inc.</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>Chief Executive Officer Arbor Biotechnologies, Inc.
-Dr. Devyn Smith brings significant cell and gene therapy development and platform expertise from his 20+ year career. Devyn joined Arbor Biotechnologies as Chief Executive Officer on April 27, 2021 after concluding his role as Chief Operating Officer of Sigilon Therapeutics. Prior to Sigilon, Dr. Smith worked in a variety of roles at Pfizer Inc., including COO of the UK-based Neusentis Unit focused on discovering and developing cell therapies. He received his Ph.D. in Genetics from Harvard Medical School. He is an inventor on multiple patents and has published in leading scientific journals throughout his career. Dr. Smith is a board member and officer for ARM (Alliance for Regenerative Medicine), the cell and gene therapy industry group
-We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
-Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
-This website uses the following types of services. Learn more from our
-                    Cookie Policy.
-By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>https://genetherapy-conference.com/speaker/devyn-smith/</t>
-        </is>
-      </c>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>https://genetherapy-conference.com/wp-content/uploads/sites/227/2025/11/62945-Speaker-Photos-10-300x300.png</t>
-        </is>
-      </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>images/devyn_smith.jpg</t>
-        </is>
-      </c>
-      <c r="N29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>CONF-3FC9E8</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Gene Therapy Conference</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Gene Therapy</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Hebe</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>Hebe Sun</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>Associate Director, CDx/IVD Regulatory Affairs</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>Regeneron Pharmaceuticals</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>Associate Director, CDx/IVD Regulatory Affairs Regeneron Pharmaceuticals
-Hebe Sun, Regulatory Affairs Associate Director in Regeneron, contributed to the CDx/IVD co-development in multiple gene therapy programs in Regeneron. Before Regeneron, she has multiple years of regulatory experience in medical device and IVD industry.
-We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
-Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
-This website uses the following types of services. Learn more from our
-                    Cookie Policy.
-By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>https://genetherapy-conference.com/speaker/hebe-sun/</t>
-        </is>
-      </c>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>https://genetherapy-conference.com/wp-content/uploads/sites/227/2025/11/62945-Speaker-Photos-11-300x300.png</t>
-        </is>
-      </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>images/hebe_sun.jpg</t>
-        </is>
-      </c>
-      <c r="N30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>CONF-3FC9E8</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Gene Therapy Conference</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Gene Therapy</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>Tassos</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>Tassos Georgiadis</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>Senior VP, Discovery &amp; Preclinical Development</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>MeiraGTx</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>Senior VP, Discovery &amp; Preclinical Development MeiraGTx
-Tassos has been working on retinal gene therapy for 25 years. He has developed AAV vectors for a range of indications that are currently in clinical development (Ph1/2, Ph3, pre-commercialization). He is currently Senior Vice President, Discovery &amp; Preclinical Development at MeiraGTx establishing a multi-platform assessment strategy for drug product candidate screening, with a focus on retina and CNS.
-We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
-Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
-This website uses the following types of services. Learn more from our
-                    Cookie Policy.
-By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>https://genetherapy-conference.com/speaker/tassos-georgiadis/</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>https://genetherapy-conference.com/wp-content/uploads/sites/227/2025/11/62945-Speaker-Photos-27-300x300.png</t>
-        </is>
-      </c>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>images/tassos_georgiadis.jpg</t>
-        </is>
-      </c>
-      <c r="N31" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>CONF-3FC9E8</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Gene Therapy Conference</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Gene Therapy</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>Casey</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>Casey Maguire</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>Investigator &amp; Associate Professor</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>Harvard Medical School</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>Investigator &amp; Associate Professor Harvard Medical School
-Casey A. Maguire obtained a B.S. in Microbiology from the University of Maine in 2000 and a PhD from the Department of Microbiology and Immunology at the University of Rochester School of Medicine and Dentistry in 2006. He was a postdoctoral fellow at the MGH from 2006-2010. He was next an Instructor from 2010-2013 and Assistant Professor from 2013-2019. Currently he is an Associate Professor of Neurology at Harvard Medical School with his laboratory located at the MGH Research Institute.
-We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
-Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
-This website uses the following types of services. Learn more from our
-                    Cookie Policy.
-By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
-        </is>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>https://genetherapy-conference.com/speaker/casey-maguire/</t>
-        </is>
-      </c>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>https://genetherapy-conference.com/wp-content/uploads/sites/227/2025/11/62945-Speaker-Photos-4-300x300.png</t>
-        </is>
-      </c>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>images/casey_maguire.jpg</t>
-        </is>
-      </c>
-      <c r="N32" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>CONF-3FC9E8</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Gene Therapy Conference</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Gene Therapy</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>Lindsay</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>Lindsay Marjoram</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>CSO</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>Barth Syndrome Foundation Inc</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>Lindsay Marjoram, PhD is the Director of Research for the Barth Syndrome Foundation, which is dedicated to advocacy and advancing research for the development of treatments and, one day, cures for this ultra-rare disease. Dr. Marjoram has a background in developmental biology and a vested interest in rare disease research. Prior to joining the Barth Syndrome Foundation, Dr. Marjoram worked for a pre-clinical contract research organization specialized in ophthalmology where she gained extensive experience in cutting edge gene therapies and rare diseases impacting vision loss
-We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
-Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
-This website uses the following types of services. Learn more from our
-                    Cookie Policy.
-By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>https://genetherapy-conference.com/speaker/lindsay-marjoram/</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>https://genetherapy-conference.com/wp-content/uploads/sites/227/2025/11/62945-Speaker-Photos-16-300x300.png</t>
-        </is>
-      </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>images/lindsay_marjoram.jpg</t>
-        </is>
-      </c>
-      <c r="N33" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>CONF-3FC9E8</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Gene Therapy Conference</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Gene Therapy</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>Susan</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>Susan serrano</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>Senior Director, Market Access Strategy and Value Communication</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>Intellia Therapeutics</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>Senior Director, Market Access Strategy and Value Communication Intellia Therapeutics
-We are always looking for ambitious people to join our team. You'll have opportunities to learn quickly, advance your career, and to meaningfully impact our customers and our business.
-Hanson Wade specializes in scientific research across a comprehensive range of distinctive R&amp;D areas. We deliver insight and connections to facilitate safe and effective drug development for more personalized and targeted patient populations.
-This website uses the following types of services. Learn more from our
-                    Cookie Policy.
-By clicking “opt out”, the browser on this device will be opted out of sharing personal data.</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>https://genetherapy-conference.com/speaker/susan-serrano/</t>
-        </is>
-      </c>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>https://genetherapy-conference.com/wp-content/uploads/sites/227/2025/11/Susan-Serrano-300x300.png</t>
-        </is>
-      </c>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>images/susan_serrano.jpg</t>
-        </is>
-      </c>
-      <c r="N34" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
added logic to extract dates and location from websites
</commit_message>
<xml_diff>
--- a/conference_data.xlsx
+++ b/conference_data.xlsx
@@ -506,12 +506,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>April 2026</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -570,12 +570,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>April 2026</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -634,12 +634,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>April 2026</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -698,12 +698,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>April 2026</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -762,12 +762,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>April 2026</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -830,12 +830,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>April 2026</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -894,12 +894,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>April 2026</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -958,12 +958,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>April 2026</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1022,12 +1022,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>April 2026</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1082,12 +1082,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>April 2026</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1146,12 +1146,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>April, 2027</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>London, UK</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1210,12 +1210,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>April, 2027</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>London, UK</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1274,12 +1274,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>April, 2027</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>London, UK</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1344,12 +1344,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>April, 2027</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>London, UK</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1408,12 +1408,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>April, 2027</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>London, UK</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1474,12 +1474,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>April, 2027</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>London, UK</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1539,12 +1539,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>April, 2027</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>London, UK</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1603,12 +1603,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>April, 2027</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>London, UK</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1667,12 +1667,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>June 2-4, 2026</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1731,12 +1731,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>June 2-4, 2026</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1796,12 +1796,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>June 2-4, 2026</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1860,12 +1860,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>June 2-4, 2026</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1920,12 +1920,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>June 2-4, 2026</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1985,12 +1985,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>June 2-4, 2026</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2053,12 +2053,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>June 2-4, 2026</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Boston, MA</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">

</xml_diff>